<commit_message>
add amistoso vs Nazca individual 37mi, corregir tiro por pase
</commit_message>
<xml_diff>
--- a/events.xlsx
+++ b/events.xlsx
@@ -5,11 +5,13 @@
   <sheets>
     <sheet state="visible" name="Hoja1" sheetId="1" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">Hoja1!$A$1:$O$304</definedName>
+  </definedNames>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="OH/cYb2NQ1tMXHiXbMdcNOJkNg9nu1bwMkfH3ZyVEBI="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="Z3NMd00D7vcHXh3a2P1rbUboFcvMRm78Oa2XFCzdNzc="/>
     </ext>
   </extLst>
 </workbook>
@@ -777,6 +779,9 @@
     <t xml:space="preserve">91;18 97;41 </t>
   </si>
   <si>
+    <t>TIRO</t>
+  </si>
+  <si>
     <t>06:39</t>
   </si>
   <si>
@@ -1123,9 +1128,6 @@
   </si>
   <si>
     <t xml:space="preserve">71;77 69;63 </t>
-  </si>
-  <si>
-    <t>TIRO</t>
   </si>
   <si>
     <t>09:58</t>
@@ -3217,7 +3219,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -3225,12 +3227,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <sz val="10.0"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -3238,12 +3240,9 @@
       <name val="Arial"/>
     </font>
     <font>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <u/>
       <color rgb="FF0000FF"/>
+      <name val="Roboto"/>
     </font>
     <font>
       <color rgb="FF434343"/>
@@ -3436,31 +3435,39 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="45">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="49" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="3" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -3471,11 +3478,11 @@
     <xf borderId="5" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="5" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="5" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="6" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="6" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -3486,12 +3493,14 @@
     <xf borderId="2" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="3" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -3499,13 +3508,15 @@
     <xf borderId="5" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="5" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="5" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="6" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="6" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="3" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -3518,16 +3529,29 @@
     <xf borderId="8" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="5" fillId="3" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="6" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="6" fillId="3" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="2" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="0"/>
+    <xf borderId="6" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="5" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="0"/>
+    <xf borderId="4" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="4" fontId="3" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="9" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -3538,18 +3562,20 @@
     <xf borderId="10" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="10" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="10" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="10" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="11" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="10" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="11" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="5">
     <dxf>
       <font/>
       <fill>
@@ -3561,8 +3587,8 @@
       <font/>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
+          <fgColor rgb="FF356854"/>
+          <bgColor rgb="FF356854"/>
         </patternFill>
       </fill>
       <border/>
@@ -3571,18 +3597,45 @@
       <font/>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="0"/>
-          <bgColor theme="0"/>
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
         </patternFill>
       </fill>
       <border/>
     </dxf>
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="3" pivot="0" name="Hoja1-style">
+    <tableStyle count="4" pivot="0" name="Hoja1-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="2" type="secondRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
   </tableStyles>
 </styleSheet>
@@ -3593,7 +3646,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:O304" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:O304" displayName="Tabla_1" name="Tabla_1" id="1">
+  <autoFilter ref="$A$1:$O$304">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="PASE"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="15">
     <tableColumn name="Event" id="1"/>
     <tableColumn name="start_time" id="2"/>
@@ -3875,7 +3935,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" ht="12.75" customHeight="1">
+    <row r="2" ht="12.75" hidden="1" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>15</v>
       </c>
@@ -3912,7 +3972,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" ht="12.75" customHeight="1">
+    <row r="3" ht="12.75" hidden="1" customHeight="1">
       <c r="A3" s="11" t="s">
         <v>15</v>
       </c>
@@ -3949,7 +4009,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="12.75" customHeight="1">
+    <row r="4" ht="12.75" hidden="1" customHeight="1">
       <c r="A4" s="16" t="s">
         <v>15</v>
       </c>
@@ -3986,7 +4046,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" ht="12.75" customHeight="1">
+    <row r="5" ht="12.75" hidden="1" customHeight="1">
       <c r="A5" s="22" t="s">
         <v>15</v>
       </c>
@@ -4023,7 +4083,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" ht="12.75" customHeight="1">
+    <row r="6" ht="12.75" hidden="1" customHeight="1">
       <c r="A6" s="16" t="s">
         <v>15</v>
       </c>
@@ -4060,7 +4120,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" ht="12.75" customHeight="1">
+    <row r="7" ht="12.75" hidden="1" customHeight="1">
       <c r="A7" s="22" t="s">
         <v>15</v>
       </c>
@@ -4097,7 +4157,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" ht="12.75" customHeight="1">
+    <row r="8" ht="12.75" hidden="1" customHeight="1">
       <c r="A8" s="16" t="s">
         <v>15</v>
       </c>
@@ -4134,7 +4194,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" ht="12.75" customHeight="1">
+    <row r="9" ht="12.75" hidden="1" customHeight="1">
       <c r="A9" s="22" t="s">
         <v>15</v>
       </c>
@@ -4171,7 +4231,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" ht="12.75" customHeight="1">
+    <row r="10" ht="12.75" hidden="1" customHeight="1">
       <c r="A10" s="16" t="s">
         <v>50</v>
       </c>
@@ -4210,7 +4270,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" ht="12.75" customHeight="1">
+    <row r="11" ht="12.75" hidden="1" customHeight="1">
       <c r="A11" s="22" t="s">
         <v>15</v>
       </c>
@@ -4247,7 +4307,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" ht="12.75" customHeight="1">
+    <row r="12" ht="12.75" hidden="1" customHeight="1">
       <c r="A12" s="28" t="s">
         <v>15</v>
       </c>
@@ -4284,7 +4344,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" ht="12.75" customHeight="1">
+    <row r="13" ht="12.75" hidden="1" customHeight="1">
       <c r="A13" s="22" t="s">
         <v>15</v>
       </c>
@@ -4321,7 +4381,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" ht="12.75" customHeight="1">
+    <row r="14" ht="12.75" hidden="1" customHeight="1">
       <c r="A14" s="16" t="s">
         <v>15</v>
       </c>
@@ -4358,7 +4418,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" ht="12.75" customHeight="1">
+    <row r="15" ht="12.75" hidden="1" customHeight="1">
       <c r="A15" s="22" t="s">
         <v>50</v>
       </c>
@@ -4395,7 +4455,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" ht="12.75" customHeight="1">
+    <row r="16" ht="12.75" hidden="1" customHeight="1">
       <c r="A16" s="28" t="s">
         <v>15</v>
       </c>
@@ -4432,7 +4492,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" ht="12.75" customHeight="1">
+    <row r="17" ht="12.75" hidden="1" customHeight="1">
       <c r="A17" s="22" t="s">
         <v>15</v>
       </c>
@@ -4469,7 +4529,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" ht="12.75" customHeight="1">
+    <row r="18" ht="12.75" hidden="1" customHeight="1">
       <c r="A18" s="16" t="s">
         <v>15</v>
       </c>
@@ -4506,7 +4566,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" ht="12.75" customHeight="1">
+    <row r="19" ht="12.75" hidden="1" customHeight="1">
       <c r="A19" s="22" t="s">
         <v>88</v>
       </c>
@@ -4623,7 +4683,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" ht="12.75" customHeight="1">
+    <row r="22" ht="12.75" hidden="1" customHeight="1">
       <c r="A22" s="16" t="s">
         <v>99</v>
       </c>
@@ -4664,7 +4724,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" ht="12.75" customHeight="1">
+    <row r="23" ht="12.75" hidden="1" customHeight="1">
       <c r="A23" s="22" t="s">
         <v>99</v>
       </c>
@@ -4705,7 +4765,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" ht="12.75" customHeight="1">
+    <row r="24" ht="12.75" hidden="1" customHeight="1">
       <c r="A24" s="16" t="s">
         <v>99</v>
       </c>
@@ -4746,7 +4806,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" ht="12.75" customHeight="1">
+    <row r="25" ht="12.75" hidden="1" customHeight="1">
       <c r="A25" s="22" t="s">
         <v>99</v>
       </c>
@@ -4826,7 +4886,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" ht="12.75" customHeight="1">
+    <row r="27" ht="12.75" hidden="1" customHeight="1">
       <c r="A27" s="22" t="s">
         <v>15</v>
       </c>
@@ -4863,7 +4923,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" ht="12.75" customHeight="1">
+    <row r="28" ht="12.75" hidden="1" customHeight="1">
       <c r="A28" s="16" t="s">
         <v>119</v>
       </c>
@@ -4902,7 +4962,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" ht="12.75" customHeight="1">
+    <row r="29" ht="12.75" hidden="1" customHeight="1">
       <c r="A29" s="22" t="s">
         <v>119</v>
       </c>
@@ -4941,7 +5001,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" ht="12.75" customHeight="1">
+    <row r="30" ht="12.75" hidden="1" customHeight="1">
       <c r="A30" s="16" t="s">
         <v>128</v>
       </c>
@@ -5101,7 +5161,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" ht="12.75" customHeight="1">
+    <row r="34" ht="12.75" hidden="1" customHeight="1">
       <c r="A34" s="16" t="s">
         <v>141</v>
       </c>
@@ -5179,7 +5239,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" ht="12.75" customHeight="1">
+    <row r="36" ht="12.75" hidden="1" customHeight="1">
       <c r="A36" s="16" t="s">
         <v>15</v>
       </c>
@@ -5503,7 +5563,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="44" ht="12.75" customHeight="1">
+    <row r="44" ht="12.75" hidden="1" customHeight="1">
       <c r="A44" s="16" t="s">
         <v>99</v>
       </c>
@@ -5544,7 +5604,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="45" ht="12.75" customHeight="1">
+    <row r="45" ht="12.75" hidden="1" customHeight="1">
       <c r="A45" s="22" t="s">
         <v>99</v>
       </c>
@@ -5626,7 +5686,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="47" ht="12.75" customHeight="1">
+    <row r="47" ht="12.75" hidden="1" customHeight="1">
       <c r="A47" s="22" t="s">
         <v>188</v>
       </c>
@@ -5663,7 +5723,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="48" ht="12.75" customHeight="1">
+    <row r="48" ht="12.75" hidden="1" customHeight="1">
       <c r="A48" s="16" t="s">
         <v>99</v>
       </c>
@@ -5704,7 +5764,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="49" ht="12.75" customHeight="1">
+    <row r="49" ht="12.75" hidden="1" customHeight="1">
       <c r="A49" s="22" t="s">
         <v>15</v>
       </c>
@@ -5741,7 +5801,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="50" ht="12.75" customHeight="1">
+    <row r="50" ht="12.75" hidden="1" customHeight="1">
       <c r="A50" s="16" t="s">
         <v>15</v>
       </c>
@@ -5778,7 +5838,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="51" ht="12.75" customHeight="1">
+    <row r="51" ht="12.75" hidden="1" customHeight="1">
       <c r="A51" s="22" t="s">
         <v>15</v>
       </c>
@@ -5815,7 +5875,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="52" ht="12.75" customHeight="1">
+    <row r="52" ht="12.75" hidden="1" customHeight="1">
       <c r="A52" s="16" t="s">
         <v>208</v>
       </c>
@@ -6018,7 +6078,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="57" ht="12.75" customHeight="1">
+    <row r="57" ht="12.75" hidden="1" customHeight="1">
       <c r="A57" s="22" t="s">
         <v>141</v>
       </c>
@@ -6180,7 +6240,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="61" ht="12.75" customHeight="1">
+    <row r="61" ht="12.75" hidden="1" customHeight="1">
       <c r="A61" s="22" t="s">
         <v>128</v>
       </c>
@@ -6342,7 +6402,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="65" ht="12.75" customHeight="1">
+    <row r="65" ht="12.75" hidden="1" customHeight="1">
       <c r="A65" s="22" t="s">
         <v>141</v>
       </c>
@@ -6423,20 +6483,20 @@
       </c>
     </row>
     <row r="67" ht="12.75" customHeight="1">
-      <c r="A67" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="B67" s="12" t="s">
+      <c r="A67" s="34" t="s">
         <v>253</v>
       </c>
-      <c r="C67" s="12" t="s">
+      <c r="B67" s="35" t="s">
         <v>254</v>
       </c>
-      <c r="D67" s="12" t="s">
+      <c r="C67" s="35" t="s">
         <v>255</v>
       </c>
-      <c r="E67" s="23" t="s">
+      <c r="D67" s="35" t="s">
         <v>256</v>
+      </c>
+      <c r="E67" s="36" t="s">
+        <v>257</v>
       </c>
       <c r="F67" s="24"/>
       <c r="G67" s="23" t="s">
@@ -6461,21 +6521,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="68" ht="12.75" customHeight="1">
+    <row r="68" ht="12.75" hidden="1" customHeight="1">
       <c r="A68" s="16" t="s">
         <v>188</v>
       </c>
       <c r="B68" s="17" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C68" s="17" t="s">
         <v>248</v>
       </c>
       <c r="D68" s="17" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E68" s="18" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F68" s="19"/>
       <c r="G68" s="19"/>
@@ -6498,21 +6558,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="69" ht="12.75" customHeight="1">
+    <row r="69" ht="12.75" hidden="1" customHeight="1">
       <c r="A69" s="22" t="s">
         <v>15</v>
       </c>
       <c r="B69" s="12" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D69" s="12" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E69" s="23" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F69" s="24"/>
       <c r="G69" s="24"/>
@@ -6535,21 +6595,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="70" ht="12.75" customHeight="1">
+    <row r="70" ht="12.75" hidden="1" customHeight="1">
       <c r="A70" s="16" t="s">
         <v>119</v>
       </c>
       <c r="B70" s="17" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C70" s="17" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D70" s="17" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E70" s="18" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F70" s="19"/>
       <c r="G70" s="18" t="s">
@@ -6579,16 +6639,16 @@
         <v>92</v>
       </c>
       <c r="B71" s="12" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D71" s="12" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E71" s="23" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F71" s="24"/>
       <c r="G71" s="23" t="s">
@@ -6615,21 +6675,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="72" ht="12.75" customHeight="1">
+    <row r="72" ht="12.75" hidden="1" customHeight="1">
       <c r="A72" s="16" t="s">
         <v>188</v>
       </c>
       <c r="B72" s="17" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C72" s="17" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D72" s="17" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E72" s="18" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F72" s="19"/>
       <c r="G72" s="19"/>
@@ -6652,21 +6712,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="73" ht="12.75" customHeight="1">
+    <row r="73" ht="12.75" hidden="1" customHeight="1">
       <c r="A73" s="22" t="s">
         <v>119</v>
       </c>
       <c r="B73" s="12" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D73" s="12" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E73" s="23" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F73" s="24"/>
       <c r="G73" s="23" t="s">
@@ -6691,21 +6751,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="74" ht="12.75" customHeight="1">
+    <row r="74" ht="12.75" hidden="1" customHeight="1">
       <c r="A74" s="16" t="s">
         <v>15</v>
       </c>
       <c r="B74" s="17" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C74" s="17" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D74" s="17" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E74" s="18" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F74" s="19"/>
       <c r="G74" s="19"/>
@@ -6728,21 +6788,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="75" ht="12.75" customHeight="1">
+    <row r="75" ht="12.75" hidden="1" customHeight="1">
       <c r="A75" s="22" t="s">
         <v>15</v>
       </c>
       <c r="B75" s="12" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C75" s="12" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D75" s="12" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F75" s="24"/>
       <c r="G75" s="24"/>
@@ -6765,21 +6825,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="76" ht="12.75" customHeight="1">
+    <row r="76" ht="12.75" hidden="1" customHeight="1">
       <c r="A76" s="16" t="s">
         <v>15</v>
       </c>
       <c r="B76" s="17" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C76" s="17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D76" s="17" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E76" s="18" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F76" s="19"/>
       <c r="G76" s="19"/>
@@ -6802,21 +6862,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="77" ht="12.75" customHeight="1">
+    <row r="77" ht="12.75" hidden="1" customHeight="1">
       <c r="A77" s="22" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B77" s="12" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D77" s="12" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F77" s="24"/>
       <c r="G77" s="24"/>
@@ -6825,7 +6885,7 @@
         <v>20</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K77" s="24"/>
       <c r="L77" s="25"/>
@@ -6839,24 +6899,24 @@
         <v>24</v>
       </c>
     </row>
-    <row r="78" ht="12.75" customHeight="1">
+    <row r="78" ht="12.75" hidden="1" customHeight="1">
       <c r="A78" s="16" t="s">
         <v>99</v>
       </c>
       <c r="B78" s="17" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C78" s="17" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D78" s="17" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E78" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F78" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G78" s="18" t="s">
         <v>96</v>
@@ -6885,16 +6945,16 @@
         <v>92</v>
       </c>
       <c r="B79" s="12" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D79" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F79" s="24"/>
       <c r="G79" s="23" t="s">
@@ -6921,21 +6981,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="80" ht="12.75" customHeight="1">
+    <row r="80" ht="12.75" hidden="1" customHeight="1">
       <c r="A80" s="16" t="s">
         <v>128</v>
       </c>
       <c r="B80" s="17" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C80" s="17" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D80" s="17" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E80" s="18" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F80" s="19"/>
       <c r="G80" s="18" t="s">
@@ -6960,21 +7020,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="81" ht="12.75" customHeight="1">
+    <row r="81" ht="12.75" hidden="1" customHeight="1">
       <c r="A81" s="22" t="s">
         <v>188</v>
       </c>
       <c r="B81" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D81" s="12" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F81" s="24"/>
       <c r="G81" s="24"/>
@@ -6997,21 +7057,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="82" ht="12.75" customHeight="1">
+    <row r="82" ht="12.75" hidden="1" customHeight="1">
       <c r="A82" s="16" t="s">
         <v>15</v>
       </c>
       <c r="B82" s="17" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C82" s="17" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D82" s="17" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E82" s="18" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F82" s="19"/>
       <c r="G82" s="19"/>
@@ -7034,21 +7094,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="83" ht="12.75" customHeight="1">
+    <row r="83" ht="12.75" hidden="1" customHeight="1">
       <c r="A83" s="22" t="s">
         <v>15</v>
       </c>
       <c r="B83" s="12" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C83" s="12" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D83" s="12" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E83" s="23" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F83" s="24"/>
       <c r="G83" s="24"/>
@@ -7071,21 +7131,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="84" ht="12.75" customHeight="1">
+    <row r="84" ht="12.75" hidden="1" customHeight="1">
       <c r="A84" s="16" t="s">
         <v>15</v>
       </c>
       <c r="B84" s="17" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C84" s="17" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D84" s="17" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E84" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F84" s="19"/>
       <c r="G84" s="19"/>
@@ -7108,21 +7168,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="85" ht="12.75" customHeight="1">
+    <row r="85" ht="12.75" hidden="1" customHeight="1">
       <c r="A85" s="22" t="s">
         <v>15</v>
       </c>
       <c r="B85" s="12" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C85" s="12" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D85" s="12" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E85" s="23" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F85" s="24"/>
       <c r="G85" s="24"/>
@@ -7145,21 +7205,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" ht="12.75" customHeight="1">
+    <row r="86" ht="12.75" hidden="1" customHeight="1">
       <c r="A86" s="16" t="s">
         <v>208</v>
       </c>
       <c r="B86" s="17" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C86" s="17" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D86" s="17" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E86" s="18" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F86" s="19"/>
       <c r="G86" s="19"/>
@@ -7182,21 +7242,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="87" ht="12.75" customHeight="1">
+    <row r="87" ht="12.75" hidden="1" customHeight="1">
       <c r="A87" s="22" t="s">
         <v>99</v>
       </c>
       <c r="B87" s="12" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C87" s="12" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D87" s="12" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E87" s="23" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F87" s="23" t="s">
         <v>107</v>
@@ -7223,21 +7283,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="88" ht="12.75" customHeight="1">
+    <row r="88" ht="12.75" hidden="1" customHeight="1">
       <c r="A88" s="16" t="s">
         <v>141</v>
       </c>
       <c r="B88" s="17" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C88" s="17" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D88" s="17" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E88" s="18" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F88" s="19"/>
       <c r="G88" s="19"/>
@@ -7265,16 +7325,16 @@
         <v>92</v>
       </c>
       <c r="B89" s="12" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D89" s="12" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E89" s="23" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F89" s="24"/>
       <c r="G89" s="23" t="s">
@@ -7306,16 +7366,16 @@
         <v>92</v>
       </c>
       <c r="B90" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C90" s="17" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D90" s="17" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E90" s="18" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F90" s="19"/>
       <c r="G90" s="18" t="s">
@@ -7347,16 +7407,16 @@
         <v>92</v>
       </c>
       <c r="B91" s="12" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C91" s="12" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D91" s="12" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E91" s="23" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F91" s="24"/>
       <c r="G91" s="23" t="s">
@@ -7388,16 +7448,16 @@
         <v>92</v>
       </c>
       <c r="B92" s="17" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C92" s="17" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D92" s="17" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E92" s="18" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F92" s="19"/>
       <c r="G92" s="18" t="s">
@@ -7429,16 +7489,16 @@
         <v>92</v>
       </c>
       <c r="B93" s="12" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C93" s="12" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D93" s="12" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E93" s="23" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F93" s="24"/>
       <c r="G93" s="23" t="s">
@@ -7465,21 +7525,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="94" ht="12.75" customHeight="1">
+    <row r="94" ht="12.75" hidden="1" customHeight="1">
       <c r="A94" s="16" t="s">
         <v>50</v>
       </c>
       <c r="B94" s="17" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C94" s="17" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D94" s="17" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E94" s="18" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F94" s="19"/>
       <c r="G94" s="19"/>
@@ -7502,21 +7562,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="95" ht="12.75" customHeight="1">
+    <row r="95" ht="12.75" hidden="1" customHeight="1">
       <c r="A95" s="22" t="s">
         <v>15</v>
       </c>
       <c r="B95" s="12" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C95" s="12" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D95" s="12" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E95" s="23" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F95" s="24"/>
       <c r="G95" s="24"/>
@@ -7539,21 +7599,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="96" ht="12.75" customHeight="1">
+    <row r="96" ht="12.75" hidden="1" customHeight="1">
       <c r="A96" s="16" t="s">
         <v>15</v>
       </c>
       <c r="B96" s="17" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C96" s="17" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D96" s="17" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E96" s="18" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F96" s="19"/>
       <c r="G96" s="19"/>
@@ -7576,21 +7636,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="97" ht="12.75" customHeight="1">
+    <row r="97" ht="12.75" hidden="1" customHeight="1">
       <c r="A97" s="22" t="s">
         <v>88</v>
       </c>
       <c r="B97" s="12" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C97" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D97" s="12" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E97" s="23" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F97" s="24"/>
       <c r="G97" s="23" t="s">
@@ -7620,16 +7680,16 @@
         <v>92</v>
       </c>
       <c r="B98" s="17" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C98" s="17" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D98" s="17" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E98" s="18" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F98" s="19"/>
       <c r="G98" s="18" t="s">
@@ -7661,16 +7721,16 @@
         <v>92</v>
       </c>
       <c r="B99" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C99" s="12" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D99" s="12" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E99" s="23" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F99" s="24"/>
       <c r="G99" s="23" t="s">
@@ -7702,16 +7762,16 @@
         <v>92</v>
       </c>
       <c r="B100" s="17" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C100" s="17" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D100" s="17" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E100" s="18" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F100" s="19"/>
       <c r="G100" s="18" t="s">
@@ -7738,15 +7798,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="101" ht="12.75" customHeight="1">
+    <row r="101" ht="12.75" hidden="1" customHeight="1">
       <c r="A101" s="22" t="s">
-        <v>369</v>
+        <v>253</v>
       </c>
       <c r="B101" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C101" s="12" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D101" s="12" t="s">
         <v>370</v>
@@ -7777,7 +7837,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="102" ht="12.75" customHeight="1">
+    <row r="102" ht="12.75" hidden="1" customHeight="1">
       <c r="A102" s="16" t="s">
         <v>119</v>
       </c>
@@ -7816,7 +7876,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="103" ht="12.75" customHeight="1">
+    <row r="103" ht="12.75" hidden="1" customHeight="1">
       <c r="A103" s="22" t="s">
         <v>15</v>
       </c>
@@ -7853,7 +7913,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="104" ht="12.75" customHeight="1">
+    <row r="104" ht="12.75" hidden="1" customHeight="1">
       <c r="A104" s="16" t="s">
         <v>50</v>
       </c>
@@ -7890,7 +7950,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="105" ht="12.75" customHeight="1">
+    <row r="105" ht="12.75" hidden="1" customHeight="1">
       <c r="A105" s="22" t="s">
         <v>15</v>
       </c>
@@ -7927,7 +7987,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="106" ht="12.75" customHeight="1">
+    <row r="106" ht="12.75" hidden="1" customHeight="1">
       <c r="A106" s="16" t="s">
         <v>15</v>
       </c>
@@ -7964,7 +8024,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="107" ht="12.75" customHeight="1">
+    <row r="107" ht="12.75" hidden="1" customHeight="1">
       <c r="A107" s="22" t="s">
         <v>15</v>
       </c>
@@ -8001,7 +8061,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="108" ht="12.75" customHeight="1">
+    <row r="108" ht="12.75" hidden="1" customHeight="1">
       <c r="A108" s="16" t="s">
         <v>88</v>
       </c>
@@ -8038,7 +8098,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="109" ht="12.75" customHeight="1">
+    <row r="109" ht="12.75" hidden="1" customHeight="1">
       <c r="A109" s="22" t="s">
         <v>396</v>
       </c>
@@ -8102,7 +8162,7 @@
         <v>20</v>
       </c>
       <c r="J110" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K110" s="18" t="s">
         <v>174</v>
@@ -8159,7 +8219,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="112" ht="12.75" customHeight="1">
+    <row r="112" ht="12.75" hidden="1" customHeight="1">
       <c r="A112" s="16" t="s">
         <v>99</v>
       </c>
@@ -8239,7 +8299,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="114" ht="12.75" customHeight="1">
+    <row r="114" ht="12.75" hidden="1" customHeight="1">
       <c r="A114" s="16" t="s">
         <v>15</v>
       </c>
@@ -8276,7 +8336,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="115" ht="12.75" customHeight="1">
+    <row r="115" ht="12.75" hidden="1" customHeight="1">
       <c r="A115" s="22" t="s">
         <v>15</v>
       </c>
@@ -8313,7 +8373,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="116" ht="12.75" customHeight="1">
+    <row r="116" ht="12.75" hidden="1" customHeight="1">
       <c r="A116" s="16" t="s">
         <v>99</v>
       </c>
@@ -8339,7 +8399,7 @@
       <c r="I116" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J116" s="34" t="s">
+      <c r="J116" s="37" t="s">
         <v>76</v>
       </c>
       <c r="K116" s="19"/>
@@ -8354,7 +8414,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="117" ht="12.75" customHeight="1">
+    <row r="117" ht="12.75" hidden="1" customHeight="1">
       <c r="A117" s="22" t="s">
         <v>15</v>
       </c>
@@ -8391,7 +8451,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="118" ht="12.75" customHeight="1">
+    <row r="118" ht="12.75" hidden="1" customHeight="1">
       <c r="A118" s="16" t="s">
         <v>15</v>
       </c>
@@ -8428,7 +8488,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="119" ht="12.75" customHeight="1">
+    <row r="119" ht="12.75" hidden="1" customHeight="1">
       <c r="A119" s="22" t="s">
         <v>99</v>
       </c>
@@ -8454,7 +8514,7 @@
       <c r="I119" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J119" s="35" t="s">
+      <c r="J119" s="38" t="s">
         <v>34</v>
       </c>
       <c r="K119" s="24"/>
@@ -8469,9 +8529,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="120" ht="12.75" customHeight="1">
+    <row r="120" ht="12.75" hidden="1" customHeight="1">
       <c r="A120" s="16" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B120" s="17" t="s">
         <v>437</v>
@@ -8506,7 +8566,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="121" ht="12.75" customHeight="1">
+    <row r="121" ht="12.75" hidden="1" customHeight="1">
       <c r="A121" s="22" t="s">
         <v>396</v>
       </c>
@@ -8573,7 +8633,7 @@
         <v>76</v>
       </c>
       <c r="K122" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L122" s="21"/>
       <c r="M122" s="7" t="s">
@@ -8611,7 +8671,7 @@
         <v>20</v>
       </c>
       <c r="J123" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K123" s="23" t="s">
         <v>174</v>
@@ -8653,7 +8713,7 @@
         <v>174</v>
       </c>
       <c r="K124" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L124" s="21"/>
       <c r="M124" s="7" t="s">
@@ -8691,7 +8751,7 @@
         <v>20</v>
       </c>
       <c r="J125" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K125" s="23" t="s">
         <v>211</v>
@@ -8735,7 +8795,7 @@
         <v>211</v>
       </c>
       <c r="K126" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L126" s="21"/>
       <c r="M126" s="7" t="s">
@@ -8773,7 +8833,7 @@
         <v>20</v>
       </c>
       <c r="J127" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K127" s="23" t="s">
         <v>71</v>
@@ -8871,7 +8931,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="130" ht="12.75" customHeight="1">
+    <row r="130" ht="12.75" hidden="1" customHeight="1">
       <c r="A130" s="16" t="s">
         <v>141</v>
       </c>
@@ -9139,7 +9199,7 @@
         <v>123</v>
       </c>
       <c r="K136" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L136" s="21"/>
       <c r="M136" s="7" t="s">
@@ -9177,7 +9237,7 @@
         <v>20</v>
       </c>
       <c r="J137" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K137" s="23" t="s">
         <v>123</v>
@@ -9271,7 +9331,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="140" ht="12.75" customHeight="1">
+    <row r="140" ht="12.75" hidden="1" customHeight="1">
       <c r="A140" s="16" t="s">
         <v>99</v>
       </c>
@@ -9295,7 +9355,7 @@
       <c r="I140" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J140" s="34" t="s">
+      <c r="J140" s="37" t="s">
         <v>34</v>
       </c>
       <c r="K140" s="19"/>
@@ -9420,7 +9480,7 @@
         <v>174</v>
       </c>
       <c r="K143" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L143" s="25"/>
       <c r="M143" s="7" t="s">
@@ -9458,7 +9518,7 @@
         <v>20</v>
       </c>
       <c r="J144" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K144" s="19"/>
       <c r="L144" s="21"/>
@@ -9472,7 +9532,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="145" ht="12.75" customHeight="1">
+    <row r="145" ht="12.75" hidden="1" customHeight="1">
       <c r="A145" s="22" t="s">
         <v>15</v>
       </c>
@@ -9509,7 +9569,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="146" ht="12.75" customHeight="1">
+    <row r="146" ht="12.75" hidden="1" customHeight="1">
       <c r="A146" s="16" t="s">
         <v>50</v>
       </c>
@@ -9546,9 +9606,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="147" ht="12.75" customHeight="1">
+    <row r="147" ht="12.75" hidden="1" customHeight="1">
       <c r="A147" s="22" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B147" s="12" t="s">
         <v>528</v>
@@ -9583,7 +9643,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="148" ht="12.75" customHeight="1">
+    <row r="148" ht="12.75" hidden="1" customHeight="1">
       <c r="A148" s="16" t="s">
         <v>141</v>
       </c>
@@ -9620,9 +9680,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="149" ht="12.75" customHeight="1">
+    <row r="149" ht="12.75" hidden="1" customHeight="1">
       <c r="A149" s="22" t="s">
-        <v>369</v>
+        <v>253</v>
       </c>
       <c r="B149" s="12" t="s">
         <v>529</v>
@@ -9659,7 +9719,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="150" ht="12.75" customHeight="1">
+    <row r="150" ht="12.75" hidden="1" customHeight="1">
       <c r="A150" s="16" t="s">
         <v>15</v>
       </c>
@@ -9696,7 +9756,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="151" ht="12.75" customHeight="1">
+    <row r="151" ht="12.75" hidden="1" customHeight="1">
       <c r="A151" s="22" t="s">
         <v>15</v>
       </c>
@@ -9763,7 +9823,7 @@
         <v>211</v>
       </c>
       <c r="K152" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L152" s="21"/>
       <c r="M152" s="7" t="s">
@@ -9801,7 +9861,7 @@
         <v>20</v>
       </c>
       <c r="J153" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K153" s="23" t="s">
         <v>211</v>
@@ -9856,7 +9916,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="155" ht="12.75" customHeight="1">
+    <row r="155" ht="12.75" hidden="1" customHeight="1">
       <c r="A155" s="22" t="s">
         <v>99</v>
       </c>
@@ -9878,7 +9938,7 @@
       <c r="I155" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J155" s="35" t="s">
+      <c r="J155" s="38" t="s">
         <v>62</v>
       </c>
       <c r="K155" s="24"/>
@@ -9893,7 +9953,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="156" ht="12.75" customHeight="1">
+    <row r="156" ht="12.75" hidden="1" customHeight="1">
       <c r="A156" s="16" t="s">
         <v>99</v>
       </c>
@@ -9919,7 +9979,7 @@
       <c r="I156" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J156" s="34" t="s">
+      <c r="J156" s="37" t="s">
         <v>62</v>
       </c>
       <c r="K156" s="19"/>
@@ -9934,7 +9994,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="157" ht="12.75" customHeight="1">
+    <row r="157" ht="12.75" hidden="1" customHeight="1">
       <c r="A157" s="22" t="s">
         <v>88</v>
       </c>
@@ -10096,7 +10156,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="161" ht="12.75" customHeight="1">
+    <row r="161" ht="12.75" hidden="1" customHeight="1">
       <c r="A161" s="22" t="s">
         <v>141</v>
       </c>
@@ -10284,7 +10344,7 @@
         <v>123</v>
       </c>
       <c r="K165" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L165" s="25"/>
       <c r="M165" s="7" t="s">
@@ -10322,7 +10382,7 @@
         <v>20</v>
       </c>
       <c r="J166" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K166" s="18" t="s">
         <v>76</v>
@@ -10377,7 +10437,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="168" ht="12.75" customHeight="1">
+    <row r="168" ht="12.75" hidden="1" customHeight="1">
       <c r="A168" s="16" t="s">
         <v>88</v>
       </c>
@@ -10457,7 +10517,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="170" ht="12.75" customHeight="1">
+    <row r="170" ht="12.75" hidden="1" customHeight="1">
       <c r="A170" s="16" t="s">
         <v>128</v>
       </c>
@@ -10496,7 +10556,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="171" ht="12.75" customHeight="1">
+    <row r="171" ht="12.75" hidden="1" customHeight="1">
       <c r="A171" s="22" t="s">
         <v>141</v>
       </c>
@@ -10576,7 +10636,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="173" ht="12.75" customHeight="1">
+    <row r="173" ht="12.75" hidden="1" customHeight="1">
       <c r="A173" s="22" t="s">
         <v>188</v>
       </c>
@@ -10613,9 +10673,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="174" ht="12.75" customHeight="1">
+    <row r="174" ht="12.75" hidden="1" customHeight="1">
       <c r="A174" s="16" t="s">
-        <v>369</v>
+        <v>253</v>
       </c>
       <c r="B174" s="17" t="s">
         <v>601</v>
@@ -10654,7 +10714,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="175" ht="12.75" customHeight="1">
+    <row r="175" ht="12.75" hidden="1" customHeight="1">
       <c r="A175" s="22" t="s">
         <v>15</v>
       </c>
@@ -10691,9 +10751,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="176" ht="12.75" customHeight="1">
+    <row r="176" ht="12.75" hidden="1" customHeight="1">
       <c r="A176" s="16" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B176" s="17" t="s">
         <v>619</v>
@@ -10728,7 +10788,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="177" ht="12.75" customHeight="1">
+    <row r="177" ht="12.75" hidden="1" customHeight="1">
       <c r="A177" s="22" t="s">
         <v>15</v>
       </c>
@@ -10765,7 +10825,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="178" ht="12.75" customHeight="1">
+    <row r="178" ht="12.75" hidden="1" customHeight="1">
       <c r="A178" s="16" t="s">
         <v>15</v>
       </c>
@@ -10802,7 +10862,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="179" ht="12.75" customHeight="1">
+    <row r="179" ht="12.75" hidden="1" customHeight="1">
       <c r="A179" s="22" t="s">
         <v>15</v>
       </c>
@@ -10839,7 +10899,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="180" ht="12.75" customHeight="1">
+    <row r="180" ht="12.75" hidden="1" customHeight="1">
       <c r="A180" s="16" t="s">
         <v>15</v>
       </c>
@@ -10876,7 +10936,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="181" ht="12.75" customHeight="1">
+    <row r="181" ht="12.75" hidden="1" customHeight="1">
       <c r="A181" s="22" t="s">
         <v>15</v>
       </c>
@@ -10913,7 +10973,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="182" ht="12.75" customHeight="1">
+    <row r="182" ht="12.75" hidden="1" customHeight="1">
       <c r="A182" s="16" t="s">
         <v>15</v>
       </c>
@@ -10950,7 +11010,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="183" ht="12.75" customHeight="1">
+    <row r="183" ht="12.75" hidden="1" customHeight="1">
       <c r="A183" s="22" t="s">
         <v>88</v>
       </c>
@@ -11071,7 +11131,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="186" ht="12.75" customHeight="1">
+    <row r="186" ht="12.75" hidden="1" customHeight="1">
       <c r="A186" s="16" t="s">
         <v>141</v>
       </c>
@@ -11108,9 +11168,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="187" ht="12.75" customHeight="1">
+    <row r="187" ht="12.75" hidden="1" customHeight="1">
       <c r="A187" s="22" t="s">
-        <v>369</v>
+        <v>253</v>
       </c>
       <c r="B187" s="12" t="s">
         <v>661</v>
@@ -11147,7 +11207,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="188" ht="12.75" customHeight="1">
+    <row r="188" ht="12.75" hidden="1" customHeight="1">
       <c r="A188" s="16" t="s">
         <v>15</v>
       </c>
@@ -11184,7 +11244,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="189" ht="12.75" customHeight="1">
+    <row r="189" ht="12.75" hidden="1" customHeight="1">
       <c r="A189" s="22" t="s">
         <v>15</v>
       </c>
@@ -11221,7 +11281,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="190" ht="12.75" customHeight="1">
+    <row r="190" ht="12.75" hidden="1" customHeight="1">
       <c r="A190" s="16" t="s">
         <v>128</v>
       </c>
@@ -11260,7 +11320,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="191" ht="12.75" customHeight="1">
+    <row r="191" ht="12.75" hidden="1" customHeight="1">
       <c r="A191" s="22" t="s">
         <v>396</v>
       </c>
@@ -11327,7 +11387,7 @@
         <v>76</v>
       </c>
       <c r="K192" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L192" s="21"/>
       <c r="M192" s="7" t="s">
@@ -11365,7 +11425,7 @@
         <v>20</v>
       </c>
       <c r="J193" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K193" s="23" t="s">
         <v>211</v>
@@ -11409,7 +11469,7 @@
         <v>211</v>
       </c>
       <c r="K194" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L194" s="21"/>
       <c r="M194" s="7" t="s">
@@ -11450,7 +11510,7 @@
         <v>71</v>
       </c>
       <c r="K195" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L195" s="25"/>
       <c r="M195" s="7" t="s">
@@ -11666,7 +11726,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="201" ht="12.75" customHeight="1">
+    <row r="201" ht="12.75" hidden="1" customHeight="1">
       <c r="A201" s="22" t="s">
         <v>15</v>
       </c>
@@ -11703,7 +11763,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="202" ht="12.75" customHeight="1">
+    <row r="202" ht="12.75" hidden="1" customHeight="1">
       <c r="A202" s="16" t="s">
         <v>88</v>
       </c>
@@ -11768,7 +11828,7 @@
         <v>174</v>
       </c>
       <c r="K203" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L203" s="25"/>
       <c r="M203" s="7" t="s">
@@ -11806,7 +11866,7 @@
         <v>20</v>
       </c>
       <c r="J204" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K204" s="18" t="s">
         <v>71</v>
@@ -11822,7 +11882,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="205" ht="12.75" customHeight="1">
+    <row r="205" ht="12.75" hidden="1" customHeight="1">
       <c r="A205" s="22" t="s">
         <v>141</v>
       </c>
@@ -11941,9 +12001,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="208" ht="12.75" customHeight="1">
+    <row r="208" ht="12.75" hidden="1" customHeight="1">
       <c r="A208" s="16" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B208" s="17" t="s">
         <v>732</v>
@@ -11978,7 +12038,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="209" ht="12.75" customHeight="1">
+    <row r="209" ht="12.75" hidden="1" customHeight="1">
       <c r="A209" s="22" t="s">
         <v>15</v>
       </c>
@@ -12015,7 +12075,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="210" ht="12.75" customHeight="1">
+    <row r="210" ht="12.75" hidden="1" customHeight="1">
       <c r="A210" s="16" t="s">
         <v>99</v>
       </c>
@@ -12032,7 +12092,7 @@
         <v>740</v>
       </c>
       <c r="F210" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G210" s="18" t="s">
         <v>98</v>
@@ -12056,7 +12116,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="211" ht="12.75" customHeight="1">
+    <row r="211" ht="12.75" hidden="1" customHeight="1">
       <c r="A211" s="22" t="s">
         <v>50</v>
       </c>
@@ -12093,7 +12153,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="212" ht="12.75" customHeight="1">
+    <row r="212" ht="12.75" hidden="1" customHeight="1">
       <c r="A212" s="16" t="s">
         <v>15</v>
       </c>
@@ -12130,9 +12190,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="213" ht="12.75" customHeight="1">
+    <row r="213" ht="12.75" hidden="1" customHeight="1">
       <c r="A213" s="22" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B213" s="12" t="s">
         <v>749</v>
@@ -12167,7 +12227,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="214" ht="12.75" customHeight="1">
+    <row r="214" ht="12.75" hidden="1" customHeight="1">
       <c r="A214" s="16" t="s">
         <v>99</v>
       </c>
@@ -12194,7 +12254,7 @@
         <v>20</v>
       </c>
       <c r="J214" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K214" s="26"/>
       <c r="L214" s="21"/>
@@ -12372,7 +12432,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="219" ht="12.75" customHeight="1">
+    <row r="219" ht="12.75" hidden="1" customHeight="1">
       <c r="A219" s="22" t="s">
         <v>141</v>
       </c>
@@ -12450,7 +12510,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="221" ht="12.75" customHeight="1">
+    <row r="221" ht="12.75" hidden="1" customHeight="1">
       <c r="A221" s="22" t="s">
         <v>141</v>
       </c>
@@ -12487,7 +12547,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="222" ht="12.75" customHeight="1">
+    <row r="222" ht="12.75" hidden="1" customHeight="1">
       <c r="A222" s="16" t="s">
         <v>99</v>
       </c>
@@ -12528,7 +12588,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="223" ht="12.75" customHeight="1">
+    <row r="223" ht="12.75" hidden="1" customHeight="1">
       <c r="A223" s="22" t="s">
         <v>15</v>
       </c>
@@ -12565,7 +12625,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="224" ht="12.75" customHeight="1">
+    <row r="224" ht="12.75" hidden="1" customHeight="1">
       <c r="A224" s="16" t="s">
         <v>119</v>
       </c>
@@ -12606,7 +12666,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="225" ht="12.75" customHeight="1">
+    <row r="225" ht="12.75" hidden="1" customHeight="1">
       <c r="A225" s="22" t="s">
         <v>15</v>
       </c>
@@ -12643,7 +12703,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="226" ht="12.75" customHeight="1">
+    <row r="226" ht="12.75" hidden="1" customHeight="1">
       <c r="A226" s="16" t="s">
         <v>15</v>
       </c>
@@ -12680,7 +12740,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="227" ht="12.75" customHeight="1">
+    <row r="227" ht="12.75" hidden="1" customHeight="1">
       <c r="A227" s="22" t="s">
         <v>119</v>
       </c>
@@ -12719,7 +12779,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="228" ht="12.75" customHeight="1">
+    <row r="228" ht="12.75" hidden="1" customHeight="1">
       <c r="A228" s="16" t="s">
         <v>15</v>
       </c>
@@ -12756,7 +12816,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="229" ht="12.75" customHeight="1">
+    <row r="229" ht="12.75" hidden="1" customHeight="1">
       <c r="A229" s="22" t="s">
         <v>15</v>
       </c>
@@ -12793,7 +12853,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="230" ht="12.75" customHeight="1">
+    <row r="230" ht="12.75" hidden="1" customHeight="1">
       <c r="A230" s="16" t="s">
         <v>119</v>
       </c>
@@ -12832,7 +12892,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="231" ht="12.75" customHeight="1">
+    <row r="231" ht="12.75" hidden="1" customHeight="1">
       <c r="A231" s="22" t="s">
         <v>208</v>
       </c>
@@ -12846,7 +12906,7 @@
         <v>814</v>
       </c>
       <c r="E231" s="23" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F231" s="24"/>
       <c r="G231" s="24"/>
@@ -12869,7 +12929,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="232" ht="12.75" customHeight="1">
+    <row r="232" ht="12.75" hidden="1" customHeight="1">
       <c r="A232" s="16" t="s">
         <v>15</v>
       </c>
@@ -12906,7 +12966,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="233" ht="12.75" customHeight="1">
+    <row r="233" ht="12.75" hidden="1" customHeight="1">
       <c r="A233" s="22" t="s">
         <v>15</v>
       </c>
@@ -12943,7 +13003,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="234" ht="12.75" customHeight="1">
+    <row r="234" ht="12.75" hidden="1" customHeight="1">
       <c r="A234" s="16" t="s">
         <v>15</v>
       </c>
@@ -12980,7 +13040,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="235" ht="12.75" customHeight="1">
+    <row r="235" ht="12.75" hidden="1" customHeight="1">
       <c r="A235" s="22" t="s">
         <v>15</v>
       </c>
@@ -13017,7 +13077,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="236" ht="12.75" customHeight="1">
+    <row r="236" ht="12.75" hidden="1" customHeight="1">
       <c r="A236" s="16" t="s">
         <v>15</v>
       </c>
@@ -13040,7 +13100,7 @@
         <v>20</v>
       </c>
       <c r="J236" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K236" s="19"/>
       <c r="L236" s="21"/>
@@ -13054,7 +13114,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="237" ht="12.75" customHeight="1">
+    <row r="237" ht="12.75" hidden="1" customHeight="1">
       <c r="A237" s="22" t="s">
         <v>141</v>
       </c>
@@ -13130,7 +13190,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="239" ht="12.75" customHeight="1">
+    <row r="239" ht="12.75" hidden="1" customHeight="1">
       <c r="A239" s="22" t="s">
         <v>88</v>
       </c>
@@ -13292,7 +13352,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="243" ht="12.75" customHeight="1">
+    <row r="243" ht="12.75" hidden="1" customHeight="1">
       <c r="A243" s="22" t="s">
         <v>141</v>
       </c>
@@ -13329,7 +13389,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="244" ht="12.75" customHeight="1">
+    <row r="244" ht="12.75" hidden="1" customHeight="1">
       <c r="A244" s="16" t="s">
         <v>99</v>
       </c>
@@ -13368,7 +13428,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="245" ht="12.75" customHeight="1">
+    <row r="245" ht="12.75" hidden="1" customHeight="1">
       <c r="A245" s="22" t="s">
         <v>119</v>
       </c>
@@ -13407,9 +13467,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="246" ht="12.75" customHeight="1">
+    <row r="246" ht="12.75" hidden="1" customHeight="1">
       <c r="A246" s="16" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B246" s="17" t="s">
         <v>868</v>
@@ -13430,7 +13490,7 @@
         <v>20</v>
       </c>
       <c r="J246" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K246" s="19"/>
       <c r="L246" s="21"/>
@@ -13444,7 +13504,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="247" ht="12.75" customHeight="1">
+    <row r="247" ht="12.75" hidden="1" customHeight="1">
       <c r="A247" s="22" t="s">
         <v>15</v>
       </c>
@@ -13481,7 +13541,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="248" ht="12.75" customHeight="1">
+    <row r="248" ht="12.75" hidden="1" customHeight="1">
       <c r="A248" s="16" t="s">
         <v>99</v>
       </c>
@@ -13498,7 +13558,7 @@
         <v>878</v>
       </c>
       <c r="F248" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G248" s="18" t="s">
         <v>96</v>
@@ -13522,7 +13582,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="249" ht="12.75" customHeight="1">
+    <row r="249" ht="12.75" hidden="1" customHeight="1">
       <c r="A249" s="22" t="s">
         <v>15</v>
       </c>
@@ -13559,7 +13619,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="250" ht="12.75" customHeight="1">
+    <row r="250" ht="12.75" hidden="1" customHeight="1">
       <c r="A250" s="16" t="s">
         <v>119</v>
       </c>
@@ -13598,7 +13658,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="251" ht="12.75" customHeight="1">
+    <row r="251" ht="12.75" hidden="1" customHeight="1">
       <c r="A251" s="22" t="s">
         <v>15</v>
       </c>
@@ -13635,7 +13695,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="252" ht="12.75" customHeight="1">
+    <row r="252" ht="12.75" hidden="1" customHeight="1">
       <c r="A252" s="16" t="s">
         <v>88</v>
       </c>
@@ -13715,7 +13775,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="254" ht="12.75" customHeight="1">
+    <row r="254" ht="12.75" hidden="1" customHeight="1">
       <c r="A254" s="16" t="s">
         <v>141</v>
       </c>
@@ -13916,7 +13976,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="259" ht="12.75" customHeight="1">
+    <row r="259" ht="12.75" hidden="1" customHeight="1">
       <c r="A259" s="22" t="s">
         <v>99</v>
       </c>
@@ -13957,7 +14017,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="260" ht="12.75" customHeight="1">
+    <row r="260" ht="12.75" hidden="1" customHeight="1">
       <c r="A260" s="16" t="s">
         <v>119</v>
       </c>
@@ -14160,9 +14220,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="265" ht="12.75" customHeight="1">
+    <row r="265" ht="12.75" hidden="1" customHeight="1">
       <c r="A265" s="22" t="s">
-        <v>369</v>
+        <v>253</v>
       </c>
       <c r="B265" s="12" t="s">
         <v>925</v>
@@ -14199,7 +14259,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="266" ht="12.75" customHeight="1">
+    <row r="266" ht="12.75" hidden="1" customHeight="1">
       <c r="A266" s="16" t="s">
         <v>15</v>
       </c>
@@ -14385,7 +14445,7 @@
         <v>123</v>
       </c>
       <c r="K270" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L270" s="21"/>
       <c r="M270" s="7" t="s">
@@ -14423,7 +14483,7 @@
         <v>20</v>
       </c>
       <c r="J271" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K271" s="23" t="s">
         <v>211</v>
@@ -14478,7 +14538,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="273" ht="12.75" customHeight="1">
+    <row r="273" ht="12.75" hidden="1" customHeight="1">
       <c r="A273" s="22" t="s">
         <v>15</v>
       </c>
@@ -14515,7 +14575,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="274" ht="12.75" customHeight="1">
+    <row r="274" ht="12.75" hidden="1" customHeight="1">
       <c r="A274" s="16" t="s">
         <v>15</v>
       </c>
@@ -14552,7 +14612,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="275" ht="12.75" customHeight="1">
+    <row r="275" ht="12.75" hidden="1" customHeight="1">
       <c r="A275" s="22" t="s">
         <v>99</v>
       </c>
@@ -14569,7 +14629,7 @@
         <v>973</v>
       </c>
       <c r="F275" s="23" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G275" s="23" t="s">
         <v>98</v>
@@ -14593,7 +14653,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="276" ht="12.75" customHeight="1">
+    <row r="276" ht="12.75" hidden="1" customHeight="1">
       <c r="A276" s="16" t="s">
         <v>99</v>
       </c>
@@ -14610,7 +14670,7 @@
         <v>977</v>
       </c>
       <c r="F276" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G276" s="18" t="s">
         <v>98</v>
@@ -14634,7 +14694,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="277" ht="12.75" customHeight="1">
+    <row r="277" ht="12.75" hidden="1" customHeight="1">
       <c r="A277" s="22" t="s">
         <v>15</v>
       </c>
@@ -14671,7 +14731,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="278" ht="12.75" customHeight="1">
+    <row r="278" ht="12.75" hidden="1" customHeight="1">
       <c r="A278" s="16" t="s">
         <v>119</v>
       </c>
@@ -14696,7 +14756,7 @@
         <v>20</v>
       </c>
       <c r="J278" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K278" s="26"/>
       <c r="L278" s="21"/>
@@ -14792,7 +14852,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="281" ht="12.75" customHeight="1">
+    <row r="281" ht="12.75" hidden="1" customHeight="1">
       <c r="A281" s="22" t="s">
         <v>188</v>
       </c>
@@ -14829,7 +14889,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="282" ht="12.75" customHeight="1">
+    <row r="282" ht="12.75" hidden="1" customHeight="1">
       <c r="A282" s="16" t="s">
         <v>50</v>
       </c>
@@ -14866,7 +14926,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="283" ht="12.75" customHeight="1">
+    <row r="283" ht="12.75" hidden="1" customHeight="1">
       <c r="A283" s="22" t="s">
         <v>208</v>
       </c>
@@ -15135,7 +15195,7 @@
         <v>20</v>
       </c>
       <c r="J289" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K289" s="23" t="s">
         <v>211</v>
@@ -15179,7 +15239,7 @@
         <v>211</v>
       </c>
       <c r="K290" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L290" s="21"/>
       <c r="M290" s="7" t="s">
@@ -15217,7 +15277,7 @@
         <v>20</v>
       </c>
       <c r="J291" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K291" s="23" t="s">
         <v>174</v>
@@ -15302,7 +15362,7 @@
         <v>71</v>
       </c>
       <c r="K293" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L293" s="25"/>
       <c r="M293" s="7" t="s">
@@ -15340,7 +15400,7 @@
         <v>20</v>
       </c>
       <c r="J294" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K294" s="18" t="s">
         <v>71</v>
@@ -15479,7 +15539,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="298" ht="12.75" customHeight="1">
+    <row r="298" ht="12.75" hidden="1" customHeight="1">
       <c r="A298" s="16" t="s">
         <v>15</v>
       </c>
@@ -15516,7 +15576,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="299" ht="12.75" customHeight="1">
+    <row r="299" ht="12.75" hidden="1" customHeight="1">
       <c r="A299" s="22" t="s">
         <v>88</v>
       </c>
@@ -15637,7 +15697,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="302" ht="12.75" customHeight="1">
+    <row r="302" ht="12.75" hidden="1" customHeight="1">
       <c r="A302" s="16" t="s">
         <v>188</v>
       </c>
@@ -15674,7 +15734,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="303" ht="12.75" customHeight="1">
+    <row r="303" ht="12.75" hidden="1" customHeight="1">
       <c r="A303" s="22" t="s">
         <v>15</v>
       </c>
@@ -15711,35 +15771,35 @@
         <v>24</v>
       </c>
     </row>
-    <row r="304" ht="12.75" customHeight="1">
-      <c r="A304" s="36" t="s">
-        <v>369</v>
-      </c>
-      <c r="B304" s="37" t="s">
+    <row r="304" ht="12.75" hidden="1" customHeight="1">
+      <c r="A304" s="39" t="s">
+        <v>253</v>
+      </c>
+      <c r="B304" s="40" t="s">
         <v>1061</v>
       </c>
-      <c r="C304" s="37" t="s">
+      <c r="C304" s="40" t="s">
         <v>1062</v>
       </c>
-      <c r="D304" s="37" t="s">
+      <c r="D304" s="40" t="s">
         <v>1063</v>
       </c>
-      <c r="E304" s="38" t="s">
+      <c r="E304" s="41" t="s">
         <v>1064</v>
       </c>
-      <c r="F304" s="39"/>
-      <c r="G304" s="38" t="s">
+      <c r="F304" s="42"/>
+      <c r="G304" s="41" t="s">
         <v>96</v>
       </c>
       <c r="H304" s="20"/>
       <c r="I304" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J304" s="38" t="s">
+      <c r="J304" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="K304" s="40"/>
-      <c r="L304" s="41"/>
+      <c r="K304" s="43"/>
+      <c r="L304" s="44"/>
       <c r="M304" s="7" t="s">
         <v>22</v>
       </c>
@@ -15751,6 +15811,9 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations>
+    <dataValidation allowBlank="1" showDropDown="1" sqref="B2:D304"/>
+  </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="I2"/>
     <hyperlink r:id="rId2" ref="I3"/>

</xml_diff>

<commit_message>
des-filtrar PASES en excel
</commit_message>
<xml_diff>
--- a/events.xlsx
+++ b/events.xlsx
@@ -3650,13 +3650,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:O304" displayName="Tabla_1" name="Tabla_1" id="1">
-  <autoFilter ref="$A$1:$O$304">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="PASE"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="$A$1:$O$304"/>
   <tableColumns count="15">
     <tableColumn name="Event" id="1"/>
     <tableColumn name="start_time" id="2"/>
@@ -3938,7 +3932,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" ht="12.75" hidden="1" customHeight="1">
+    <row r="2" ht="12.75" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>15</v>
       </c>
@@ -3975,7 +3969,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" ht="12.75" hidden="1" customHeight="1">
+    <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="11" t="s">
         <v>15</v>
       </c>
@@ -4012,7 +4006,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="12.75" hidden="1" customHeight="1">
+    <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="16" t="s">
         <v>15</v>
       </c>
@@ -4049,7 +4043,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" ht="12.75" hidden="1" customHeight="1">
+    <row r="5" ht="12.75" customHeight="1">
       <c r="A5" s="22" t="s">
         <v>15</v>
       </c>
@@ -4086,7 +4080,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" ht="12.75" hidden="1" customHeight="1">
+    <row r="6" ht="12.75" customHeight="1">
       <c r="A6" s="16" t="s">
         <v>15</v>
       </c>
@@ -4123,7 +4117,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" ht="12.75" hidden="1" customHeight="1">
+    <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="22" t="s">
         <v>15</v>
       </c>
@@ -4160,7 +4154,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" ht="12.75" hidden="1" customHeight="1">
+    <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="16" t="s">
         <v>15</v>
       </c>
@@ -4197,7 +4191,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" ht="12.75" hidden="1" customHeight="1">
+    <row r="9" ht="12.75" customHeight="1">
       <c r="A9" s="22" t="s">
         <v>15</v>
       </c>
@@ -4234,7 +4228,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" ht="12.75" hidden="1" customHeight="1">
+    <row r="10" ht="12.75" customHeight="1">
       <c r="A10" s="16" t="s">
         <v>50</v>
       </c>
@@ -4273,7 +4267,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" ht="12.75" hidden="1" customHeight="1">
+    <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="22" t="s">
         <v>15</v>
       </c>
@@ -4310,7 +4304,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" ht="12.75" hidden="1" customHeight="1">
+    <row r="12" ht="12.75" customHeight="1">
       <c r="A12" s="28" t="s">
         <v>15</v>
       </c>
@@ -4347,7 +4341,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" ht="12.75" hidden="1" customHeight="1">
+    <row r="13" ht="12.75" customHeight="1">
       <c r="A13" s="22" t="s">
         <v>15</v>
       </c>
@@ -4384,7 +4378,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" ht="12.75" hidden="1" customHeight="1">
+    <row r="14" ht="12.75" customHeight="1">
       <c r="A14" s="16" t="s">
         <v>15</v>
       </c>
@@ -4421,7 +4415,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" ht="12.75" hidden="1" customHeight="1">
+    <row r="15" ht="12.75" customHeight="1">
       <c r="A15" s="22" t="s">
         <v>50</v>
       </c>
@@ -4458,7 +4452,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" ht="12.75" hidden="1" customHeight="1">
+    <row r="16" ht="12.75" customHeight="1">
       <c r="A16" s="28" t="s">
         <v>15</v>
       </c>
@@ -4495,7 +4489,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" ht="12.75" hidden="1" customHeight="1">
+    <row r="17" ht="12.75" customHeight="1">
       <c r="A17" s="22" t="s">
         <v>15</v>
       </c>
@@ -4532,7 +4526,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" ht="12.75" hidden="1" customHeight="1">
+    <row r="18" ht="12.75" customHeight="1">
       <c r="A18" s="16" t="s">
         <v>15</v>
       </c>
@@ -4569,7 +4563,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" ht="12.75" hidden="1" customHeight="1">
+    <row r="19" ht="12.75" customHeight="1">
       <c r="A19" s="22" t="s">
         <v>88</v>
       </c>
@@ -4690,7 +4684,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" ht="12.75" hidden="1" customHeight="1">
+    <row r="22" ht="12.75" customHeight="1">
       <c r="A22" s="16" t="s">
         <v>100</v>
       </c>
@@ -4731,7 +4725,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" ht="12.75" hidden="1" customHeight="1">
+    <row r="23" ht="12.75" customHeight="1">
       <c r="A23" s="22" t="s">
         <v>100</v>
       </c>
@@ -4772,7 +4766,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" ht="12.75" hidden="1" customHeight="1">
+    <row r="24" ht="12.75" customHeight="1">
       <c r="A24" s="16" t="s">
         <v>100</v>
       </c>
@@ -4813,7 +4807,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" ht="12.75" hidden="1" customHeight="1">
+    <row r="25" ht="12.75" customHeight="1">
       <c r="A25" s="22" t="s">
         <v>100</v>
       </c>
@@ -4895,7 +4889,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" ht="12.75" hidden="1" customHeight="1">
+    <row r="27" ht="12.75" customHeight="1">
       <c r="A27" s="22" t="s">
         <v>15</v>
       </c>
@@ -4932,7 +4926,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" ht="12.75" hidden="1" customHeight="1">
+    <row r="28" ht="12.75" customHeight="1">
       <c r="A28" s="16" t="s">
         <v>120</v>
       </c>
@@ -4971,7 +4965,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" ht="12.75" hidden="1" customHeight="1">
+    <row r="29" ht="12.75" customHeight="1">
       <c r="A29" s="22" t="s">
         <v>120</v>
       </c>
@@ -5010,7 +5004,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" ht="12.75" hidden="1" customHeight="1">
+    <row r="30" ht="12.75" customHeight="1">
       <c r="A30" s="16" t="s">
         <v>129</v>
       </c>
@@ -5176,7 +5170,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" ht="12.75" hidden="1" customHeight="1">
+    <row r="34" ht="12.75" customHeight="1">
       <c r="A34" s="16" t="s">
         <v>142</v>
       </c>
@@ -5256,7 +5250,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" ht="12.75" hidden="1" customHeight="1">
+    <row r="36" ht="12.75" customHeight="1">
       <c r="A36" s="16" t="s">
         <v>15</v>
       </c>
@@ -5594,7 +5588,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="44" ht="12.75" hidden="1" customHeight="1">
+    <row r="44" ht="12.75" customHeight="1">
       <c r="A44" s="16" t="s">
         <v>100</v>
       </c>
@@ -5635,7 +5629,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="45" ht="12.75" hidden="1" customHeight="1">
+    <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="22" t="s">
         <v>100</v>
       </c>
@@ -5719,7 +5713,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="47" ht="12.75" hidden="1" customHeight="1">
+    <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="22" t="s">
         <v>189</v>
       </c>
@@ -5756,7 +5750,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="48" ht="12.75" hidden="1" customHeight="1">
+    <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="16" t="s">
         <v>100</v>
       </c>
@@ -5797,7 +5791,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="49" ht="12.75" hidden="1" customHeight="1">
+    <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="22" t="s">
         <v>15</v>
       </c>
@@ -5834,7 +5828,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="50" ht="12.75" hidden="1" customHeight="1">
+    <row r="50" ht="12.75" customHeight="1">
       <c r="A50" s="16" t="s">
         <v>15</v>
       </c>
@@ -5871,7 +5865,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="51" ht="12.75" hidden="1" customHeight="1">
+    <row r="51" ht="12.75" customHeight="1">
       <c r="A51" s="22" t="s">
         <v>15</v>
       </c>
@@ -5908,7 +5902,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="52" ht="12.75" hidden="1" customHeight="1">
+    <row r="52" ht="12.75" customHeight="1">
       <c r="A52" s="16" t="s">
         <v>209</v>
       </c>
@@ -6119,7 +6113,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="57" ht="12.75" hidden="1" customHeight="1">
+    <row r="57" ht="12.75" customHeight="1">
       <c r="A57" s="22" t="s">
         <v>142</v>
       </c>
@@ -6287,7 +6281,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="61" ht="12.75" hidden="1" customHeight="1">
+    <row r="61" ht="12.75" customHeight="1">
       <c r="A61" s="22" t="s">
         <v>129</v>
       </c>
@@ -6455,7 +6449,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="65" ht="12.75" hidden="1" customHeight="1">
+    <row r="65" ht="12.75" customHeight="1">
       <c r="A65" s="22" t="s">
         <v>142</v>
       </c>
@@ -6578,7 +6572,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="68" ht="12.75" hidden="1" customHeight="1">
+    <row r="68" ht="12.75" customHeight="1">
       <c r="A68" s="16" t="s">
         <v>189</v>
       </c>
@@ -6615,7 +6609,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="69" ht="12.75" hidden="1" customHeight="1">
+    <row r="69" ht="12.75" customHeight="1">
       <c r="A69" s="22" t="s">
         <v>15</v>
       </c>
@@ -6652,7 +6646,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="70" ht="12.75" hidden="1" customHeight="1">
+    <row r="70" ht="12.75" customHeight="1">
       <c r="A70" s="16" t="s">
         <v>120</v>
       </c>
@@ -6734,7 +6728,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="72" ht="12.75" hidden="1" customHeight="1">
+    <row r="72" ht="12.75" customHeight="1">
       <c r="A72" s="16" t="s">
         <v>189</v>
       </c>
@@ -6771,7 +6765,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="73" ht="12.75" hidden="1" customHeight="1">
+    <row r="73" ht="12.75" customHeight="1">
       <c r="A73" s="22" t="s">
         <v>120</v>
       </c>
@@ -6810,7 +6804,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="74" ht="12.75" hidden="1" customHeight="1">
+    <row r="74" ht="12.75" customHeight="1">
       <c r="A74" s="16" t="s">
         <v>15</v>
       </c>
@@ -6847,7 +6841,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="75" ht="12.75" hidden="1" customHeight="1">
+    <row r="75" ht="12.75" customHeight="1">
       <c r="A75" s="22" t="s">
         <v>15</v>
       </c>
@@ -6884,7 +6878,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="76" ht="12.75" hidden="1" customHeight="1">
+    <row r="76" ht="12.75" customHeight="1">
       <c r="A76" s="16" t="s">
         <v>15</v>
       </c>
@@ -6921,7 +6915,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="77" ht="12.75" hidden="1" customHeight="1">
+    <row r="77" ht="12.75" customHeight="1">
       <c r="A77" s="22" t="s">
         <v>289</v>
       </c>
@@ -6958,7 +6952,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="78" ht="12.75" hidden="1" customHeight="1">
+    <row r="78" ht="12.75" customHeight="1">
       <c r="A78" s="16" t="s">
         <v>100</v>
       </c>
@@ -7042,7 +7036,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="80" ht="12.75" hidden="1" customHeight="1">
+    <row r="80" ht="12.75" customHeight="1">
       <c r="A80" s="16" t="s">
         <v>129</v>
       </c>
@@ -7081,7 +7075,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="81" ht="12.75" hidden="1" customHeight="1">
+    <row r="81" ht="12.75" customHeight="1">
       <c r="A81" s="22" t="s">
         <v>189</v>
       </c>
@@ -7118,7 +7112,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="82" ht="12.75" hidden="1" customHeight="1">
+    <row r="82" ht="12.75" customHeight="1">
       <c r="A82" s="16" t="s">
         <v>15</v>
       </c>
@@ -7155,7 +7149,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="83" ht="12.75" hidden="1" customHeight="1">
+    <row r="83" ht="12.75" customHeight="1">
       <c r="A83" s="22" t="s">
         <v>15</v>
       </c>
@@ -7192,7 +7186,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="84" ht="12.75" hidden="1" customHeight="1">
+    <row r="84" ht="12.75" customHeight="1">
       <c r="A84" s="16" t="s">
         <v>15</v>
       </c>
@@ -7229,7 +7223,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="85" ht="12.75" hidden="1" customHeight="1">
+    <row r="85" ht="12.75" customHeight="1">
       <c r="A85" s="22" t="s">
         <v>15</v>
       </c>
@@ -7266,7 +7260,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" ht="12.75" hidden="1" customHeight="1">
+    <row r="86" ht="12.75" customHeight="1">
       <c r="A86" s="16" t="s">
         <v>209</v>
       </c>
@@ -7303,7 +7297,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="87" ht="12.75" hidden="1" customHeight="1">
+    <row r="87" ht="12.75" customHeight="1">
       <c r="A87" s="22" t="s">
         <v>100</v>
       </c>
@@ -7344,7 +7338,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="88" ht="12.75" hidden="1" customHeight="1">
+    <row r="88" ht="12.75" customHeight="1">
       <c r="A88" s="16" t="s">
         <v>142</v>
       </c>
@@ -7596,7 +7590,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="94" ht="12.75" hidden="1" customHeight="1">
+    <row r="94" ht="12.75" customHeight="1">
       <c r="A94" s="16" t="s">
         <v>50</v>
       </c>
@@ -7633,7 +7627,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="95" ht="12.75" hidden="1" customHeight="1">
+    <row r="95" ht="12.75" customHeight="1">
       <c r="A95" s="22" t="s">
         <v>15</v>
       </c>
@@ -7670,7 +7664,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="96" ht="12.75" hidden="1" customHeight="1">
+    <row r="96" ht="12.75" customHeight="1">
       <c r="A96" s="16" t="s">
         <v>15</v>
       </c>
@@ -7707,7 +7701,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="97" ht="12.75" hidden="1" customHeight="1">
+    <row r="97" ht="12.75" customHeight="1">
       <c r="A97" s="22" t="s">
         <v>88</v>
       </c>
@@ -7875,7 +7869,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="101" ht="12.75" hidden="1" customHeight="1">
+    <row r="101" ht="12.75" customHeight="1">
       <c r="A101" s="22" t="s">
         <v>254</v>
       </c>
@@ -7914,7 +7908,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="102" ht="12.75" hidden="1" customHeight="1">
+    <row r="102" ht="12.75" customHeight="1">
       <c r="A102" s="16" t="s">
         <v>120</v>
       </c>
@@ -7953,7 +7947,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="103" ht="12.75" hidden="1" customHeight="1">
+    <row r="103" ht="12.75" customHeight="1">
       <c r="A103" s="22" t="s">
         <v>15</v>
       </c>
@@ -7990,7 +7984,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="104" ht="12.75" hidden="1" customHeight="1">
+    <row r="104" ht="12.75" customHeight="1">
       <c r="A104" s="16" t="s">
         <v>50</v>
       </c>
@@ -8027,7 +8021,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="105" ht="12.75" hidden="1" customHeight="1">
+    <row r="105" ht="12.75" customHeight="1">
       <c r="A105" s="22" t="s">
         <v>15</v>
       </c>
@@ -8064,7 +8058,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="106" ht="12.75" hidden="1" customHeight="1">
+    <row r="106" ht="12.75" customHeight="1">
       <c r="A106" s="16" t="s">
         <v>15</v>
       </c>
@@ -8101,7 +8095,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="107" ht="12.75" hidden="1" customHeight="1">
+    <row r="107" ht="12.75" customHeight="1">
       <c r="A107" s="22" t="s">
         <v>15</v>
       </c>
@@ -8138,7 +8132,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="108" ht="12.75" hidden="1" customHeight="1">
+    <row r="108" ht="12.75" customHeight="1">
       <c r="A108" s="16" t="s">
         <v>88</v>
       </c>
@@ -8175,7 +8169,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="109" ht="12.75" hidden="1" customHeight="1">
+    <row r="109" ht="12.75" customHeight="1">
       <c r="A109" s="22" t="s">
         <v>397</v>
       </c>
@@ -8300,7 +8294,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="112" ht="12.75" hidden="1" customHeight="1">
+    <row r="112" ht="12.75" customHeight="1">
       <c r="A112" s="16" t="s">
         <v>100</v>
       </c>
@@ -8382,7 +8376,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="114" ht="12.75" hidden="1" customHeight="1">
+    <row r="114" ht="12.75" customHeight="1">
       <c r="A114" s="16" t="s">
         <v>15</v>
       </c>
@@ -8419,7 +8413,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="115" ht="12.75" hidden="1" customHeight="1">
+    <row r="115" ht="12.75" customHeight="1">
       <c r="A115" s="22" t="s">
         <v>15</v>
       </c>
@@ -8456,7 +8450,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="116" ht="12.75" hidden="1" customHeight="1">
+    <row r="116" ht="12.75" customHeight="1">
       <c r="A116" s="16" t="s">
         <v>100</v>
       </c>
@@ -8497,7 +8491,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="117" ht="12.75" hidden="1" customHeight="1">
+    <row r="117" ht="12.75" customHeight="1">
       <c r="A117" s="22" t="s">
         <v>15</v>
       </c>
@@ -8534,7 +8528,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="118" ht="12.75" hidden="1" customHeight="1">
+    <row r="118" ht="12.75" customHeight="1">
       <c r="A118" s="16" t="s">
         <v>15</v>
       </c>
@@ -8571,7 +8565,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="119" ht="12.75" hidden="1" customHeight="1">
+    <row r="119" ht="12.75" customHeight="1">
       <c r="A119" s="22" t="s">
         <v>100</v>
       </c>
@@ -8612,7 +8606,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="120" ht="12.75" hidden="1" customHeight="1">
+    <row r="120" ht="12.75" customHeight="1">
       <c r="A120" s="16" t="s">
         <v>289</v>
       </c>
@@ -8649,7 +8643,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="121" ht="12.75" hidden="1" customHeight="1">
+    <row r="121" ht="12.75" customHeight="1">
       <c r="A121" s="22" t="s">
         <v>397</v>
       </c>
@@ -9030,7 +9024,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="130" ht="12.75" hidden="1" customHeight="1">
+    <row r="130" ht="12.75" customHeight="1">
       <c r="A130" s="16" t="s">
         <v>142</v>
       </c>
@@ -9448,7 +9442,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="140" ht="12.75" hidden="1" customHeight="1">
+    <row r="140" ht="12.75" customHeight="1">
       <c r="A140" s="16" t="s">
         <v>100</v>
       </c>
@@ -9657,7 +9651,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="145" ht="12.75" hidden="1" customHeight="1">
+    <row r="145" ht="12.75" customHeight="1">
       <c r="A145" s="22" t="s">
         <v>15</v>
       </c>
@@ -9694,7 +9688,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="146" ht="12.75" hidden="1" customHeight="1">
+    <row r="146" ht="12.75" customHeight="1">
       <c r="A146" s="16" t="s">
         <v>50</v>
       </c>
@@ -9731,7 +9725,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="147" ht="12.75" hidden="1" customHeight="1">
+    <row r="147" ht="12.75" customHeight="1">
       <c r="A147" s="22" t="s">
         <v>289</v>
       </c>
@@ -9768,7 +9762,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="148" ht="12.75" hidden="1" customHeight="1">
+    <row r="148" ht="12.75" customHeight="1">
       <c r="A148" s="16" t="s">
         <v>142</v>
       </c>
@@ -9805,7 +9799,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="149" ht="12.75" hidden="1" customHeight="1">
+    <row r="149" ht="12.75" customHeight="1">
       <c r="A149" s="22" t="s">
         <v>254</v>
       </c>
@@ -9844,7 +9838,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="150" ht="12.75" hidden="1" customHeight="1">
+    <row r="150" ht="12.75" customHeight="1">
       <c r="A150" s="16" t="s">
         <v>15</v>
       </c>
@@ -9881,7 +9875,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="151" ht="12.75" hidden="1" customHeight="1">
+    <row r="151" ht="12.75" customHeight="1">
       <c r="A151" s="22" t="s">
         <v>15</v>
       </c>
@@ -10047,7 +10041,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="155" ht="12.75" hidden="1" customHeight="1">
+    <row r="155" ht="12.75" customHeight="1">
       <c r="A155" s="22" t="s">
         <v>100</v>
       </c>
@@ -10084,7 +10078,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="156" ht="12.75" hidden="1" customHeight="1">
+    <row r="156" ht="12.75" customHeight="1">
       <c r="A156" s="16" t="s">
         <v>100</v>
       </c>
@@ -10125,7 +10119,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="157" ht="12.75" hidden="1" customHeight="1">
+    <row r="157" ht="12.75" customHeight="1">
       <c r="A157" s="22" t="s">
         <v>88</v>
       </c>
@@ -10293,7 +10287,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="161" ht="12.75" hidden="1" customHeight="1">
+    <row r="161" ht="12.75" customHeight="1">
       <c r="A161" s="22" t="s">
         <v>142</v>
       </c>
@@ -10586,7 +10580,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="168" ht="12.75" hidden="1" customHeight="1">
+    <row r="168" ht="12.75" customHeight="1">
       <c r="A168" s="16" t="s">
         <v>88</v>
       </c>
@@ -10668,7 +10662,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="170" ht="12.75" hidden="1" customHeight="1">
+    <row r="170" ht="12.75" customHeight="1">
       <c r="A170" s="16" t="s">
         <v>129</v>
       </c>
@@ -10707,7 +10701,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="171" ht="12.75" hidden="1" customHeight="1">
+    <row r="171" ht="12.75" customHeight="1">
       <c r="A171" s="22" t="s">
         <v>142</v>
       </c>
@@ -10789,7 +10783,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="173" ht="12.75" hidden="1" customHeight="1">
+    <row r="173" ht="12.75" customHeight="1">
       <c r="A173" s="22" t="s">
         <v>189</v>
       </c>
@@ -10826,7 +10820,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="174" ht="12.75" hidden="1" customHeight="1">
+    <row r="174" ht="12.75" customHeight="1">
       <c r="A174" s="16" t="s">
         <v>254</v>
       </c>
@@ -10867,7 +10861,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="175" ht="12.75" hidden="1" customHeight="1">
+    <row r="175" ht="12.75" customHeight="1">
       <c r="A175" s="22" t="s">
         <v>15</v>
       </c>
@@ -10904,7 +10898,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="176" ht="12.75" hidden="1" customHeight="1">
+    <row r="176" ht="12.75" customHeight="1">
       <c r="A176" s="16" t="s">
         <v>289</v>
       </c>
@@ -10941,7 +10935,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="177" ht="12.75" hidden="1" customHeight="1">
+    <row r="177" ht="12.75" customHeight="1">
       <c r="A177" s="22" t="s">
         <v>15</v>
       </c>
@@ -10978,7 +10972,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="178" ht="12.75" hidden="1" customHeight="1">
+    <row r="178" ht="12.75" customHeight="1">
       <c r="A178" s="16" t="s">
         <v>15</v>
       </c>
@@ -11015,7 +11009,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="179" ht="12.75" hidden="1" customHeight="1">
+    <row r="179" ht="12.75" customHeight="1">
       <c r="A179" s="22" t="s">
         <v>15</v>
       </c>
@@ -11052,7 +11046,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="180" ht="12.75" hidden="1" customHeight="1">
+    <row r="180" ht="12.75" customHeight="1">
       <c r="A180" s="16" t="s">
         <v>15</v>
       </c>
@@ -11089,7 +11083,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="181" ht="12.75" hidden="1" customHeight="1">
+    <row r="181" ht="12.75" customHeight="1">
       <c r="A181" s="22" t="s">
         <v>15</v>
       </c>
@@ -11126,7 +11120,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="182" ht="12.75" hidden="1" customHeight="1">
+    <row r="182" ht="12.75" customHeight="1">
       <c r="A182" s="16" t="s">
         <v>15</v>
       </c>
@@ -11163,7 +11157,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="183" ht="12.75" hidden="1" customHeight="1">
+    <row r="183" ht="12.75" customHeight="1">
       <c r="A183" s="22" t="s">
         <v>88</v>
       </c>
@@ -11288,7 +11282,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="186" ht="12.75" hidden="1" customHeight="1">
+    <row r="186" ht="12.75" customHeight="1">
       <c r="A186" s="16" t="s">
         <v>142</v>
       </c>
@@ -11325,7 +11319,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="187" ht="12.75" hidden="1" customHeight="1">
+    <row r="187" ht="12.75" customHeight="1">
       <c r="A187" s="22" t="s">
         <v>254</v>
       </c>
@@ -11364,7 +11358,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="188" ht="12.75" hidden="1" customHeight="1">
+    <row r="188" ht="12.75" customHeight="1">
       <c r="A188" s="16" t="s">
         <v>15</v>
       </c>
@@ -11401,7 +11395,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="189" ht="12.75" hidden="1" customHeight="1">
+    <row r="189" ht="12.75" customHeight="1">
       <c r="A189" s="22" t="s">
         <v>15</v>
       </c>
@@ -11438,7 +11432,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="190" ht="12.75" hidden="1" customHeight="1">
+    <row r="190" ht="12.75" customHeight="1">
       <c r="A190" s="16" t="s">
         <v>129</v>
       </c>
@@ -11477,7 +11471,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="191" ht="12.75" hidden="1" customHeight="1">
+    <row r="191" ht="12.75" customHeight="1">
       <c r="A191" s="22" t="s">
         <v>397</v>
       </c>
@@ -11901,7 +11895,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="201" ht="12.75" hidden="1" customHeight="1">
+    <row r="201" ht="12.75" customHeight="1">
       <c r="A201" s="22" t="s">
         <v>15</v>
       </c>
@@ -11938,7 +11932,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="202" ht="12.75" hidden="1" customHeight="1">
+    <row r="202" ht="12.75" customHeight="1">
       <c r="A202" s="16" t="s">
         <v>88</v>
       </c>
@@ -12061,7 +12055,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="205" ht="12.75" hidden="1" customHeight="1">
+    <row r="205" ht="12.75" customHeight="1">
       <c r="A205" s="22" t="s">
         <v>142</v>
       </c>
@@ -12184,7 +12178,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="208" ht="12.75" hidden="1" customHeight="1">
+    <row r="208" ht="12.75" customHeight="1">
       <c r="A208" s="16" t="s">
         <v>289</v>
       </c>
@@ -12221,7 +12215,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="209" ht="12.75" hidden="1" customHeight="1">
+    <row r="209" ht="12.75" customHeight="1">
       <c r="A209" s="22" t="s">
         <v>15</v>
       </c>
@@ -12258,7 +12252,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="210" ht="12.75" hidden="1" customHeight="1">
+    <row r="210" ht="12.75" customHeight="1">
       <c r="A210" s="16" t="s">
         <v>100</v>
       </c>
@@ -12299,7 +12293,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="211" ht="12.75" hidden="1" customHeight="1">
+    <row r="211" ht="12.75" customHeight="1">
       <c r="A211" s="22" t="s">
         <v>50</v>
       </c>
@@ -12336,7 +12330,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="212" ht="12.75" hidden="1" customHeight="1">
+    <row r="212" ht="12.75" customHeight="1">
       <c r="A212" s="16" t="s">
         <v>15</v>
       </c>
@@ -12373,7 +12367,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="213" ht="12.75" hidden="1" customHeight="1">
+    <row r="213" ht="12.75" customHeight="1">
       <c r="A213" s="22" t="s">
         <v>289</v>
       </c>
@@ -12410,7 +12404,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="214" ht="12.75" hidden="1" customHeight="1">
+    <row r="214" ht="12.75" customHeight="1">
       <c r="A214" s="16" t="s">
         <v>100</v>
       </c>
@@ -12623,7 +12617,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="219" ht="12.75" hidden="1" customHeight="1">
+    <row r="219" ht="12.75" customHeight="1">
       <c r="A219" s="22" t="s">
         <v>142</v>
       </c>
@@ -12703,7 +12697,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="221" ht="12.75" hidden="1" customHeight="1">
+    <row r="221" ht="12.75" customHeight="1">
       <c r="A221" s="22" t="s">
         <v>142</v>
       </c>
@@ -12740,7 +12734,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="222" ht="12.75" hidden="1" customHeight="1">
+    <row r="222" ht="12.75" customHeight="1">
       <c r="A222" s="16" t="s">
         <v>100</v>
       </c>
@@ -12781,7 +12775,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="223" ht="12.75" hidden="1" customHeight="1">
+    <row r="223" ht="12.75" customHeight="1">
       <c r="A223" s="22" t="s">
         <v>15</v>
       </c>
@@ -12818,7 +12812,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="224" ht="12.75" hidden="1" customHeight="1">
+    <row r="224" ht="12.75" customHeight="1">
       <c r="A224" s="16" t="s">
         <v>120</v>
       </c>
@@ -12859,7 +12853,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="225" ht="12.75" hidden="1" customHeight="1">
+    <row r="225" ht="12.75" customHeight="1">
       <c r="A225" s="22" t="s">
         <v>15</v>
       </c>
@@ -12896,7 +12890,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="226" ht="12.75" hidden="1" customHeight="1">
+    <row r="226" ht="12.75" customHeight="1">
       <c r="A226" s="16" t="s">
         <v>15</v>
       </c>
@@ -12933,7 +12927,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="227" ht="12.75" hidden="1" customHeight="1">
+    <row r="227" ht="12.75" customHeight="1">
       <c r="A227" s="22" t="s">
         <v>120</v>
       </c>
@@ -12972,7 +12966,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="228" ht="12.75" hidden="1" customHeight="1">
+    <row r="228" ht="12.75" customHeight="1">
       <c r="A228" s="16" t="s">
         <v>15</v>
       </c>
@@ -13009,7 +13003,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="229" ht="12.75" hidden="1" customHeight="1">
+    <row r="229" ht="12.75" customHeight="1">
       <c r="A229" s="22" t="s">
         <v>15</v>
       </c>
@@ -13046,7 +13040,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="230" ht="12.75" hidden="1" customHeight="1">
+    <row r="230" ht="12.75" customHeight="1">
       <c r="A230" s="16" t="s">
         <v>120</v>
       </c>
@@ -13085,7 +13079,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="231" ht="12.75" hidden="1" customHeight="1">
+    <row r="231" ht="12.75" customHeight="1">
       <c r="A231" s="22" t="s">
         <v>209</v>
       </c>
@@ -13122,7 +13116,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="232" ht="12.75" hidden="1" customHeight="1">
+    <row r="232" ht="12.75" customHeight="1">
       <c r="A232" s="16" t="s">
         <v>15</v>
       </c>
@@ -13159,7 +13153,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="233" ht="12.75" hidden="1" customHeight="1">
+    <row r="233" ht="12.75" customHeight="1">
       <c r="A233" s="22" t="s">
         <v>15</v>
       </c>
@@ -13196,7 +13190,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="234" ht="12.75" hidden="1" customHeight="1">
+    <row r="234" ht="12.75" customHeight="1">
       <c r="A234" s="16" t="s">
         <v>15</v>
       </c>
@@ -13233,7 +13227,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="235" ht="12.75" hidden="1" customHeight="1">
+    <row r="235" ht="12.75" customHeight="1">
       <c r="A235" s="22" t="s">
         <v>15</v>
       </c>
@@ -13270,7 +13264,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="236" ht="12.75" hidden="1" customHeight="1">
+    <row r="236" ht="12.75" customHeight="1">
       <c r="A236" s="16" t="s">
         <v>15</v>
       </c>
@@ -13307,7 +13301,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="237" ht="12.75" hidden="1" customHeight="1">
+    <row r="237" ht="12.75" customHeight="1">
       <c r="A237" s="22" t="s">
         <v>142</v>
       </c>
@@ -13385,7 +13379,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="239" ht="12.75" hidden="1" customHeight="1">
+    <row r="239" ht="12.75" customHeight="1">
       <c r="A239" s="22" t="s">
         <v>88</v>
       </c>
@@ -13553,7 +13547,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="243" ht="12.75" hidden="1" customHeight="1">
+    <row r="243" ht="12.75" customHeight="1">
       <c r="A243" s="22" t="s">
         <v>142</v>
       </c>
@@ -13590,7 +13584,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="244" ht="12.75" hidden="1" customHeight="1">
+    <row r="244" ht="12.75" customHeight="1">
       <c r="A244" s="16" t="s">
         <v>100</v>
       </c>
@@ -13629,7 +13623,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="245" ht="12.75" hidden="1" customHeight="1">
+    <row r="245" ht="12.75" customHeight="1">
       <c r="A245" s="22" t="s">
         <v>120</v>
       </c>
@@ -13668,7 +13662,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="246" ht="12.75" hidden="1" customHeight="1">
+    <row r="246" ht="12.75" customHeight="1">
       <c r="A246" s="16" t="s">
         <v>289</v>
       </c>
@@ -13705,7 +13699,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="247" ht="12.75" hidden="1" customHeight="1">
+    <row r="247" ht="12.75" customHeight="1">
       <c r="A247" s="22" t="s">
         <v>15</v>
       </c>
@@ -13742,7 +13736,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="248" ht="12.75" hidden="1" customHeight="1">
+    <row r="248" ht="12.75" customHeight="1">
       <c r="A248" s="16" t="s">
         <v>100</v>
       </c>
@@ -13783,7 +13777,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="249" ht="12.75" hidden="1" customHeight="1">
+    <row r="249" ht="12.75" customHeight="1">
       <c r="A249" s="22" t="s">
         <v>15</v>
       </c>
@@ -13820,7 +13814,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="250" ht="12.75" hidden="1" customHeight="1">
+    <row r="250" ht="12.75" customHeight="1">
       <c r="A250" s="16" t="s">
         <v>120</v>
       </c>
@@ -13859,7 +13853,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="251" ht="12.75" hidden="1" customHeight="1">
+    <row r="251" ht="12.75" customHeight="1">
       <c r="A251" s="22" t="s">
         <v>15</v>
       </c>
@@ -13896,7 +13890,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="252" ht="12.75" hidden="1" customHeight="1">
+    <row r="252" ht="12.75" customHeight="1">
       <c r="A252" s="16" t="s">
         <v>88</v>
       </c>
@@ -13978,7 +13972,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="254" ht="12.75" hidden="1" customHeight="1">
+    <row r="254" ht="12.75" customHeight="1">
       <c r="A254" s="16" t="s">
         <v>142</v>
       </c>
@@ -14187,7 +14181,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="259" ht="12.75" hidden="1" customHeight="1">
+    <row r="259" ht="12.75" customHeight="1">
       <c r="A259" s="22" t="s">
         <v>100</v>
       </c>
@@ -14228,7 +14222,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="260" ht="12.75" hidden="1" customHeight="1">
+    <row r="260" ht="12.75" customHeight="1">
       <c r="A260" s="16" t="s">
         <v>120</v>
       </c>
@@ -14439,7 +14433,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="265" ht="12.75" hidden="1" customHeight="1">
+    <row r="265" ht="12.75" customHeight="1">
       <c r="A265" s="22" t="s">
         <v>254</v>
       </c>
@@ -14478,7 +14472,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="266" ht="12.75" hidden="1" customHeight="1">
+    <row r="266" ht="12.75" customHeight="1">
       <c r="A266" s="16" t="s">
         <v>15</v>
       </c>
@@ -14769,7 +14763,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="273" ht="12.75" hidden="1" customHeight="1">
+    <row r="273" ht="12.75" customHeight="1">
       <c r="A273" s="22" t="s">
         <v>15</v>
       </c>
@@ -14806,7 +14800,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="274" ht="12.75" hidden="1" customHeight="1">
+    <row r="274" ht="12.75" customHeight="1">
       <c r="A274" s="16" t="s">
         <v>15</v>
       </c>
@@ -14843,7 +14837,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="275" ht="12.75" hidden="1" customHeight="1">
+    <row r="275" ht="12.75" customHeight="1">
       <c r="A275" s="22" t="s">
         <v>100</v>
       </c>
@@ -14884,7 +14878,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="276" ht="12.75" hidden="1" customHeight="1">
+    <row r="276" ht="12.75" customHeight="1">
       <c r="A276" s="16" t="s">
         <v>100</v>
       </c>
@@ -14925,7 +14919,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="277" ht="12.75" hidden="1" customHeight="1">
+    <row r="277" ht="12.75" customHeight="1">
       <c r="A277" s="22" t="s">
         <v>15</v>
       </c>
@@ -14962,7 +14956,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="278" ht="12.75" hidden="1" customHeight="1">
+    <row r="278" ht="12.75" customHeight="1">
       <c r="A278" s="16" t="s">
         <v>120</v>
       </c>
@@ -15087,7 +15081,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="281" ht="12.75" hidden="1" customHeight="1">
+    <row r="281" ht="12.75" customHeight="1">
       <c r="A281" s="22" t="s">
         <v>189</v>
       </c>
@@ -15124,7 +15118,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="282" ht="12.75" hidden="1" customHeight="1">
+    <row r="282" ht="12.75" customHeight="1">
       <c r="A282" s="16" t="s">
         <v>50</v>
       </c>
@@ -15161,7 +15155,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="283" ht="12.75" hidden="1" customHeight="1">
+    <row r="283" ht="12.75" customHeight="1">
       <c r="A283" s="22" t="s">
         <v>209</v>
       </c>
@@ -15802,7 +15796,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="298" ht="12.75" hidden="1" customHeight="1">
+    <row r="298" ht="12.75" customHeight="1">
       <c r="A298" s="16" t="s">
         <v>15</v>
       </c>
@@ -15839,7 +15833,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="299" ht="12.75" hidden="1" customHeight="1">
+    <row r="299" ht="12.75" customHeight="1">
       <c r="A299" s="22" t="s">
         <v>88</v>
       </c>
@@ -15964,7 +15958,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="302" ht="12.75" hidden="1" customHeight="1">
+    <row r="302" ht="12.75" customHeight="1">
       <c r="A302" s="16" t="s">
         <v>189</v>
       </c>
@@ -16001,7 +15995,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="303" ht="12.75" hidden="1" customHeight="1">
+    <row r="303" ht="12.75" customHeight="1">
       <c r="A303" s="22" t="s">
         <v>15</v>
       </c>
@@ -16038,7 +16032,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="304" ht="12.75" hidden="1" customHeight="1">
+    <row r="304" ht="12.75" customHeight="1">
       <c r="A304" s="39" t="s">
         <v>254</v>
       </c>

</xml_diff>

<commit_message>
add goles 1T vs Cristal abril 2026. corregir
</commit_message>
<xml_diff>
--- a/events.xlsx
+++ b/events.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5093" uniqueCount="1435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5118" uniqueCount="1435">
   <si>
     <t>Event</t>
   </si>
@@ -18019,16 +18019,26 @@
       <c r="G316" s="54" t="s">
         <v>1082</v>
       </c>
-      <c r="H316" s="46"/>
-      <c r="I316" s="47"/>
+      <c r="H316" s="46" t="s">
+        <v>1069</v>
+      </c>
+      <c r="I316" s="47" t="s">
+        <v>1070</v>
+      </c>
       <c r="J316" s="57"/>
       <c r="K316" s="49"/>
       <c r="L316" s="55" t="s">
         <v>213</v>
       </c>
-      <c r="M316" s="51"/>
-      <c r="N316" s="10"/>
-      <c r="O316" s="46"/>
+      <c r="M316" s="51" t="s">
+        <v>23</v>
+      </c>
+      <c r="N316" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="O316" s="46" t="s">
+        <v>1072</v>
+      </c>
     </row>
     <row r="317" ht="12.75" customHeight="1">
       <c r="A317" s="55" t="s">
@@ -18052,16 +18062,26 @@
       <c r="G317" s="55" t="s">
         <v>1087</v>
       </c>
-      <c r="H317" s="46"/>
-      <c r="I317" s="47"/>
+      <c r="H317" s="46" t="s">
+        <v>1069</v>
+      </c>
+      <c r="I317" s="47" t="s">
+        <v>1070</v>
+      </c>
       <c r="J317" s="57"/>
       <c r="K317" s="49"/>
       <c r="L317" s="55" t="s">
         <v>213</v>
       </c>
-      <c r="M317" s="51"/>
-      <c r="N317" s="10"/>
-      <c r="O317" s="46"/>
+      <c r="M317" s="51" t="s">
+        <v>23</v>
+      </c>
+      <c r="N317" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="O317" s="46" t="s">
+        <v>1072</v>
+      </c>
     </row>
     <row r="318" ht="12.75" customHeight="1">
       <c r="A318" s="55" t="s">
@@ -18083,16 +18103,26 @@
       <c r="G318" s="54" t="s">
         <v>1082</v>
       </c>
-      <c r="H318" s="46"/>
-      <c r="I318" s="47"/>
+      <c r="H318" s="46" t="s">
+        <v>1069</v>
+      </c>
+      <c r="I318" s="47" t="s">
+        <v>1070</v>
+      </c>
       <c r="J318" s="57"/>
       <c r="K318" s="49"/>
       <c r="L318" s="55" t="s">
         <v>213</v>
       </c>
-      <c r="M318" s="51"/>
-      <c r="N318" s="10"/>
-      <c r="O318" s="46"/>
+      <c r="M318" s="51" t="s">
+        <v>23</v>
+      </c>
+      <c r="N318" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="O318" s="46" t="s">
+        <v>1072</v>
+      </c>
     </row>
     <row r="319" ht="12.75" customHeight="1">
       <c r="A319" s="55" t="s">
@@ -18116,16 +18146,26 @@
       <c r="G319" s="55" t="s">
         <v>1087</v>
       </c>
-      <c r="H319" s="46"/>
-      <c r="I319" s="47"/>
+      <c r="H319" s="46" t="s">
+        <v>1069</v>
+      </c>
+      <c r="I319" s="47" t="s">
+        <v>1070</v>
+      </c>
       <c r="J319" s="57"/>
       <c r="K319" s="49"/>
       <c r="L319" s="55" t="s">
         <v>213</v>
       </c>
-      <c r="M319" s="51"/>
-      <c r="N319" s="10"/>
-      <c r="O319" s="46"/>
+      <c r="M319" s="51" t="s">
+        <v>23</v>
+      </c>
+      <c r="N319" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="O319" s="46" t="s">
+        <v>1072</v>
+      </c>
     </row>
     <row r="320" ht="12.75" customHeight="1">
       <c r="A320" s="55" t="s">
@@ -18147,16 +18187,26 @@
       <c r="G320" s="54" t="s">
         <v>1082</v>
       </c>
-      <c r="H320" s="46"/>
-      <c r="I320" s="47"/>
+      <c r="H320" s="46" t="s">
+        <v>1069</v>
+      </c>
+      <c r="I320" s="47" t="s">
+        <v>1070</v>
+      </c>
       <c r="J320" s="57"/>
       <c r="K320" s="49"/>
       <c r="L320" s="55" t="s">
         <v>213</v>
       </c>
-      <c r="M320" s="51"/>
-      <c r="N320" s="10"/>
-      <c r="O320" s="46"/>
+      <c r="M320" s="51" t="s">
+        <v>23</v>
+      </c>
+      <c r="N320" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="O320" s="46" t="s">
+        <v>1072</v>
+      </c>
     </row>
     <row r="321" ht="12.75" customHeight="1">
       <c r="A321" s="52" t="s">
@@ -37820,129 +37870,134 @@
     <hyperlink r:id="rId312" ref="I313"/>
     <hyperlink r:id="rId313" ref="I314"/>
     <hyperlink r:id="rId314" ref="I315"/>
-    <hyperlink r:id="rId315" ref="I321"/>
-    <hyperlink r:id="rId316" ref="I322"/>
-    <hyperlink r:id="rId317" ref="I323"/>
-    <hyperlink r:id="rId318" ref="I324"/>
-    <hyperlink r:id="rId319" ref="I325"/>
-    <hyperlink r:id="rId320" ref="I326"/>
-    <hyperlink r:id="rId321" ref="I327"/>
-    <hyperlink r:id="rId322" ref="I328"/>
-    <hyperlink r:id="rId323" ref="I329"/>
-    <hyperlink r:id="rId324" ref="I330"/>
-    <hyperlink r:id="rId325" ref="I331"/>
-    <hyperlink r:id="rId326" ref="I332"/>
-    <hyperlink r:id="rId327" ref="I333"/>
-    <hyperlink r:id="rId328" ref="I334"/>
-    <hyperlink r:id="rId329" ref="I335"/>
-    <hyperlink r:id="rId330" ref="I336"/>
-    <hyperlink r:id="rId331" ref="I337"/>
-    <hyperlink r:id="rId332" ref="I338"/>
-    <hyperlink r:id="rId333" ref="I339"/>
-    <hyperlink r:id="rId334" ref="I340"/>
-    <hyperlink r:id="rId335" ref="I341"/>
-    <hyperlink r:id="rId336" ref="I342"/>
-    <hyperlink r:id="rId337" ref="I343"/>
-    <hyperlink r:id="rId338" ref="I344"/>
-    <hyperlink r:id="rId339" ref="I345"/>
-    <hyperlink r:id="rId340" ref="I346"/>
-    <hyperlink r:id="rId341" ref="I347"/>
-    <hyperlink r:id="rId342" ref="I348"/>
-    <hyperlink r:id="rId343" ref="I349"/>
-    <hyperlink r:id="rId344" ref="I350"/>
-    <hyperlink r:id="rId345" ref="I351"/>
-    <hyperlink r:id="rId346" ref="I352"/>
-    <hyperlink r:id="rId347" ref="I353"/>
-    <hyperlink r:id="rId348" ref="I354"/>
-    <hyperlink r:id="rId349" ref="I355"/>
-    <hyperlink r:id="rId350" ref="I356"/>
-    <hyperlink r:id="rId351" ref="I357"/>
-    <hyperlink r:id="rId352" ref="I358"/>
-    <hyperlink r:id="rId353" ref="I359"/>
-    <hyperlink r:id="rId354" ref="I360"/>
-    <hyperlink r:id="rId355" ref="I361"/>
-    <hyperlink r:id="rId356" ref="I362"/>
-    <hyperlink r:id="rId357" ref="I363"/>
-    <hyperlink r:id="rId358" ref="I364"/>
-    <hyperlink r:id="rId359" ref="I365"/>
-    <hyperlink r:id="rId360" ref="I366"/>
-    <hyperlink r:id="rId361" ref="I367"/>
-    <hyperlink r:id="rId362" ref="I368"/>
-    <hyperlink r:id="rId363" ref="I369"/>
-    <hyperlink r:id="rId364" ref="I370"/>
-    <hyperlink r:id="rId365" ref="I371"/>
-    <hyperlink r:id="rId366" ref="I372"/>
-    <hyperlink r:id="rId367" ref="I373"/>
-    <hyperlink r:id="rId368" ref="I374"/>
-    <hyperlink r:id="rId369" ref="I375"/>
-    <hyperlink r:id="rId370" ref="I376"/>
-    <hyperlink r:id="rId371" ref="I377"/>
-    <hyperlink r:id="rId372" ref="I378"/>
-    <hyperlink r:id="rId373" ref="I379"/>
-    <hyperlink r:id="rId374" ref="I380"/>
-    <hyperlink r:id="rId375" ref="I381"/>
-    <hyperlink r:id="rId376" ref="I382"/>
-    <hyperlink r:id="rId377" ref="I383"/>
-    <hyperlink r:id="rId378" ref="I384"/>
-    <hyperlink r:id="rId379" ref="I385"/>
-    <hyperlink r:id="rId380" ref="I386"/>
-    <hyperlink r:id="rId381" ref="I387"/>
-    <hyperlink r:id="rId382" ref="I388"/>
-    <hyperlink r:id="rId383" ref="I389"/>
-    <hyperlink r:id="rId384" ref="I390"/>
-    <hyperlink r:id="rId385" ref="I391"/>
-    <hyperlink r:id="rId386" ref="I392"/>
-    <hyperlink r:id="rId387" ref="I393"/>
-    <hyperlink r:id="rId388" ref="I394"/>
-    <hyperlink r:id="rId389" ref="I395"/>
-    <hyperlink r:id="rId390" ref="I396"/>
-    <hyperlink r:id="rId391" ref="I397"/>
-    <hyperlink r:id="rId392" ref="I398"/>
-    <hyperlink r:id="rId393" ref="I399"/>
-    <hyperlink r:id="rId394" ref="I400"/>
-    <hyperlink r:id="rId395" ref="I401"/>
-    <hyperlink r:id="rId396" ref="I402"/>
-    <hyperlink r:id="rId397" ref="I403"/>
-    <hyperlink r:id="rId398" ref="I404"/>
-    <hyperlink r:id="rId399" ref="I405"/>
-    <hyperlink r:id="rId400" ref="I406"/>
-    <hyperlink r:id="rId401" ref="I407"/>
-    <hyperlink r:id="rId402" ref="I408"/>
-    <hyperlink r:id="rId403" ref="I409"/>
-    <hyperlink r:id="rId404" ref="I410"/>
-    <hyperlink r:id="rId405" ref="I411"/>
-    <hyperlink r:id="rId406" ref="I412"/>
-    <hyperlink r:id="rId407" ref="I413"/>
-    <hyperlink r:id="rId408" ref="I414"/>
-    <hyperlink r:id="rId409" ref="I415"/>
-    <hyperlink r:id="rId410" ref="I416"/>
-    <hyperlink r:id="rId411" ref="I417"/>
-    <hyperlink r:id="rId412" ref="I418"/>
-    <hyperlink r:id="rId413" ref="I419"/>
-    <hyperlink r:id="rId414" ref="I420"/>
-    <hyperlink r:id="rId415" ref="I421"/>
-    <hyperlink r:id="rId416" ref="I422"/>
-    <hyperlink r:id="rId417" ref="I423"/>
-    <hyperlink r:id="rId418" ref="I424"/>
-    <hyperlink r:id="rId419" ref="I425"/>
-    <hyperlink r:id="rId420" ref="I426"/>
-    <hyperlink r:id="rId421" ref="I427"/>
-    <hyperlink r:id="rId422" ref="I428"/>
-    <hyperlink r:id="rId423" ref="I429"/>
-    <hyperlink r:id="rId424" ref="I430"/>
-    <hyperlink r:id="rId425" ref="I431"/>
-    <hyperlink r:id="rId426" ref="I432"/>
-    <hyperlink r:id="rId427" ref="I433"/>
-    <hyperlink r:id="rId428" ref="I434"/>
-    <hyperlink r:id="rId429" ref="I435"/>
-    <hyperlink r:id="rId430" ref="I436"/>
+    <hyperlink r:id="rId315" ref="I316"/>
+    <hyperlink r:id="rId316" ref="I317"/>
+    <hyperlink r:id="rId317" ref="I318"/>
+    <hyperlink r:id="rId318" ref="I319"/>
+    <hyperlink r:id="rId319" ref="I320"/>
+    <hyperlink r:id="rId320" ref="I321"/>
+    <hyperlink r:id="rId321" ref="I322"/>
+    <hyperlink r:id="rId322" ref="I323"/>
+    <hyperlink r:id="rId323" ref="I324"/>
+    <hyperlink r:id="rId324" ref="I325"/>
+    <hyperlink r:id="rId325" ref="I326"/>
+    <hyperlink r:id="rId326" ref="I327"/>
+    <hyperlink r:id="rId327" ref="I328"/>
+    <hyperlink r:id="rId328" ref="I329"/>
+    <hyperlink r:id="rId329" ref="I330"/>
+    <hyperlink r:id="rId330" ref="I331"/>
+    <hyperlink r:id="rId331" ref="I332"/>
+    <hyperlink r:id="rId332" ref="I333"/>
+    <hyperlink r:id="rId333" ref="I334"/>
+    <hyperlink r:id="rId334" ref="I335"/>
+    <hyperlink r:id="rId335" ref="I336"/>
+    <hyperlink r:id="rId336" ref="I337"/>
+    <hyperlink r:id="rId337" ref="I338"/>
+    <hyperlink r:id="rId338" ref="I339"/>
+    <hyperlink r:id="rId339" ref="I340"/>
+    <hyperlink r:id="rId340" ref="I341"/>
+    <hyperlink r:id="rId341" ref="I342"/>
+    <hyperlink r:id="rId342" ref="I343"/>
+    <hyperlink r:id="rId343" ref="I344"/>
+    <hyperlink r:id="rId344" ref="I345"/>
+    <hyperlink r:id="rId345" ref="I346"/>
+    <hyperlink r:id="rId346" ref="I347"/>
+    <hyperlink r:id="rId347" ref="I348"/>
+    <hyperlink r:id="rId348" ref="I349"/>
+    <hyperlink r:id="rId349" ref="I350"/>
+    <hyperlink r:id="rId350" ref="I351"/>
+    <hyperlink r:id="rId351" ref="I352"/>
+    <hyperlink r:id="rId352" ref="I353"/>
+    <hyperlink r:id="rId353" ref="I354"/>
+    <hyperlink r:id="rId354" ref="I355"/>
+    <hyperlink r:id="rId355" ref="I356"/>
+    <hyperlink r:id="rId356" ref="I357"/>
+    <hyperlink r:id="rId357" ref="I358"/>
+    <hyperlink r:id="rId358" ref="I359"/>
+    <hyperlink r:id="rId359" ref="I360"/>
+    <hyperlink r:id="rId360" ref="I361"/>
+    <hyperlink r:id="rId361" ref="I362"/>
+    <hyperlink r:id="rId362" ref="I363"/>
+    <hyperlink r:id="rId363" ref="I364"/>
+    <hyperlink r:id="rId364" ref="I365"/>
+    <hyperlink r:id="rId365" ref="I366"/>
+    <hyperlink r:id="rId366" ref="I367"/>
+    <hyperlink r:id="rId367" ref="I368"/>
+    <hyperlink r:id="rId368" ref="I369"/>
+    <hyperlink r:id="rId369" ref="I370"/>
+    <hyperlink r:id="rId370" ref="I371"/>
+    <hyperlink r:id="rId371" ref="I372"/>
+    <hyperlink r:id="rId372" ref="I373"/>
+    <hyperlink r:id="rId373" ref="I374"/>
+    <hyperlink r:id="rId374" ref="I375"/>
+    <hyperlink r:id="rId375" ref="I376"/>
+    <hyperlink r:id="rId376" ref="I377"/>
+    <hyperlink r:id="rId377" ref="I378"/>
+    <hyperlink r:id="rId378" ref="I379"/>
+    <hyperlink r:id="rId379" ref="I380"/>
+    <hyperlink r:id="rId380" ref="I381"/>
+    <hyperlink r:id="rId381" ref="I382"/>
+    <hyperlink r:id="rId382" ref="I383"/>
+    <hyperlink r:id="rId383" ref="I384"/>
+    <hyperlink r:id="rId384" ref="I385"/>
+    <hyperlink r:id="rId385" ref="I386"/>
+    <hyperlink r:id="rId386" ref="I387"/>
+    <hyperlink r:id="rId387" ref="I388"/>
+    <hyperlink r:id="rId388" ref="I389"/>
+    <hyperlink r:id="rId389" ref="I390"/>
+    <hyperlink r:id="rId390" ref="I391"/>
+    <hyperlink r:id="rId391" ref="I392"/>
+    <hyperlink r:id="rId392" ref="I393"/>
+    <hyperlink r:id="rId393" ref="I394"/>
+    <hyperlink r:id="rId394" ref="I395"/>
+    <hyperlink r:id="rId395" ref="I396"/>
+    <hyperlink r:id="rId396" ref="I397"/>
+    <hyperlink r:id="rId397" ref="I398"/>
+    <hyperlink r:id="rId398" ref="I399"/>
+    <hyperlink r:id="rId399" ref="I400"/>
+    <hyperlink r:id="rId400" ref="I401"/>
+    <hyperlink r:id="rId401" ref="I402"/>
+    <hyperlink r:id="rId402" ref="I403"/>
+    <hyperlink r:id="rId403" ref="I404"/>
+    <hyperlink r:id="rId404" ref="I405"/>
+    <hyperlink r:id="rId405" ref="I406"/>
+    <hyperlink r:id="rId406" ref="I407"/>
+    <hyperlink r:id="rId407" ref="I408"/>
+    <hyperlink r:id="rId408" ref="I409"/>
+    <hyperlink r:id="rId409" ref="I410"/>
+    <hyperlink r:id="rId410" ref="I411"/>
+    <hyperlink r:id="rId411" ref="I412"/>
+    <hyperlink r:id="rId412" ref="I413"/>
+    <hyperlink r:id="rId413" ref="I414"/>
+    <hyperlink r:id="rId414" ref="I415"/>
+    <hyperlink r:id="rId415" ref="I416"/>
+    <hyperlink r:id="rId416" ref="I417"/>
+    <hyperlink r:id="rId417" ref="I418"/>
+    <hyperlink r:id="rId418" ref="I419"/>
+    <hyperlink r:id="rId419" ref="I420"/>
+    <hyperlink r:id="rId420" ref="I421"/>
+    <hyperlink r:id="rId421" ref="I422"/>
+    <hyperlink r:id="rId422" ref="I423"/>
+    <hyperlink r:id="rId423" ref="I424"/>
+    <hyperlink r:id="rId424" ref="I425"/>
+    <hyperlink r:id="rId425" ref="I426"/>
+    <hyperlink r:id="rId426" ref="I427"/>
+    <hyperlink r:id="rId427" ref="I428"/>
+    <hyperlink r:id="rId428" ref="I429"/>
+    <hyperlink r:id="rId429" ref="I430"/>
+    <hyperlink r:id="rId430" ref="I431"/>
+    <hyperlink r:id="rId431" ref="I432"/>
+    <hyperlink r:id="rId432" ref="I433"/>
+    <hyperlink r:id="rId433" ref="I434"/>
+    <hyperlink r:id="rId434" ref="I435"/>
+    <hyperlink r:id="rId435" ref="I436"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <drawing r:id="rId431"/>
+  <drawing r:id="rId436"/>
   <tableParts count="1">
-    <tablePart r:id="rId433"/>
+    <tablePart r:id="rId438"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update events rival Arguedas 1T correct2
</commit_message>
<xml_diff>
--- a/events.xlsx
+++ b/events.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7828" uniqueCount="2161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7828" uniqueCount="2060">
   <si>
     <t>Event</t>
   </si>
@@ -5543,57 +5543,33 @@
     <t>Elaborado</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub19</t>
-  </si>
-  <si>
     <t>94;40</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub20</t>
-  </si>
-  <si>
     <t>02:04</t>
   </si>
   <si>
     <t>40;25</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub21</t>
-  </si>
-  <si>
-    <t>Arguedas vs Chanhas sub22</t>
-  </si>
-  <si>
     <t>02:39</t>
   </si>
   <si>
     <t>41;14</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub23</t>
-  </si>
-  <si>
     <t>13;33</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub24</t>
-  </si>
-  <si>
     <t>78;7</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub25</t>
-  </si>
-  <si>
     <t>03:47</t>
   </si>
   <si>
     <t>71;91</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub26</t>
-  </si>
-  <si>
     <t>04:03</t>
   </si>
   <si>
@@ -5603,9 +5579,6 @@
     <t>42;91</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub27</t>
-  </si>
-  <si>
     <t>04:08</t>
   </si>
   <si>
@@ -5615,9 +5588,6 @@
     <t>45;68</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub28</t>
-  </si>
-  <si>
     <t>05:03</t>
   </si>
   <si>
@@ -5627,36 +5597,24 @@
     <t>Progresiòn</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub29</t>
-  </si>
-  <si>
     <t>05:06</t>
   </si>
   <si>
     <t>43;19</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub30</t>
-  </si>
-  <si>
     <t>05:20</t>
   </si>
   <si>
     <t>41;13</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub31</t>
-  </si>
-  <si>
     <t>05:18</t>
   </si>
   <si>
     <t>77;55</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub32</t>
-  </si>
-  <si>
     <t>05:39</t>
   </si>
   <si>
@@ -5666,30 +5624,18 @@
     <t>Mixto</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub33</t>
-  </si>
-  <si>
     <t>78;88</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub34</t>
-  </si>
-  <si>
     <t>66;26</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub35</t>
-  </si>
-  <si>
     <t>06:44</t>
   </si>
   <si>
     <t>88;41</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub36</t>
-  </si>
-  <si>
     <t>06:45</t>
   </si>
   <si>
@@ -5699,33 +5645,21 @@
     <t>24;61</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub37</t>
-  </si>
-  <si>
     <t>06:58</t>
   </si>
   <si>
     <t>47;56</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub38</t>
-  </si>
-  <si>
     <t>07:27</t>
   </si>
   <si>
     <t>47;45</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub39</t>
-  </si>
-  <si>
     <t>55;81</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub40</t>
-  </si>
-  <si>
     <t>08:06</t>
   </si>
   <si>
@@ -5735,24 +5669,15 @@
     <t>87;12</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub41</t>
-  </si>
-  <si>
     <t>81;11</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub42</t>
-  </si>
-  <si>
     <t>08:33</t>
   </si>
   <si>
     <t>70;26</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub43</t>
-  </si>
-  <si>
     <t>08:56</t>
   </si>
   <si>
@@ -5762,9 +5687,6 @@
     <t>24;52</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub44</t>
-  </si>
-  <si>
     <t>09:10</t>
   </si>
   <si>
@@ -5774,27 +5696,18 @@
     <t>49;56</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub45</t>
-  </si>
-  <si>
     <t>09:23</t>
   </si>
   <si>
     <t>25;17</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub46</t>
-  </si>
-  <si>
     <t>10:02</t>
   </si>
   <si>
     <t>54;42</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub47</t>
-  </si>
-  <si>
     <t>10:04</t>
   </si>
   <si>
@@ -5804,57 +5717,36 @@
     <t>41;20</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub48</t>
-  </si>
-  <si>
     <t>10:48</t>
   </si>
   <si>
     <t>92;56</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub49</t>
-  </si>
-  <si>
     <t>46;47</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub50</t>
-  </si>
-  <si>
     <t>72;34</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub51</t>
-  </si>
-  <si>
     <t>11:21</t>
   </si>
   <si>
     <t>51;60</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub52</t>
-  </si>
-  <si>
     <t>11:22</t>
   </si>
   <si>
     <t>51;91</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub53</t>
-  </si>
-  <si>
     <t>12:24</t>
   </si>
   <si>
     <t>94;42</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub54</t>
-  </si>
-  <si>
     <t>13:00</t>
   </si>
   <si>
@@ -5864,33 +5756,21 @@
     <t>6;56</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub55</t>
-  </si>
-  <si>
     <t>98;100 95;55</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub56</t>
-  </si>
-  <si>
     <t>14:12</t>
   </si>
   <si>
     <t>95;41</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub57</t>
-  </si>
-  <si>
     <t>14:57</t>
   </si>
   <si>
     <t>45;6</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub58</t>
-  </si>
-  <si>
     <t>15:01</t>
   </si>
   <si>
@@ -5900,9 +5780,6 @@
     <t>68;28</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub59</t>
-  </si>
-  <si>
     <t>15:06</t>
   </si>
   <si>
@@ -5915,18 +5792,12 @@
     <t>51;26</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub60</t>
-  </si>
-  <si>
     <t>15:21</t>
   </si>
   <si>
     <t>68;67</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub61</t>
-  </si>
-  <si>
     <t>15:51</t>
   </si>
   <si>
@@ -5936,9 +5807,6 @@
     <t>64;50</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub62</t>
-  </si>
-  <si>
     <t>16:04</t>
   </si>
   <si>
@@ -5948,15 +5816,9 @@
     <t>17;43</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub63</t>
-  </si>
-  <si>
     <t>52;17</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub64</t>
-  </si>
-  <si>
     <t>16:28</t>
   </si>
   <si>
@@ -5966,72 +5828,45 @@
     <t>42;70</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub65</t>
-  </si>
-  <si>
     <t>17:02</t>
   </si>
   <si>
     <t>99;1 97;47</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub66</t>
-  </si>
-  <si>
     <t>17:07</t>
   </si>
   <si>
     <t>80;57</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub67</t>
-  </si>
-  <si>
     <t>9;55</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub68</t>
-  </si>
-  <si>
     <t>71;6</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub69</t>
-  </si>
-  <si>
     <t>58;28</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub70</t>
-  </si>
-  <si>
     <t>18:54</t>
   </si>
   <si>
     <t>19;83</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub71</t>
-  </si>
-  <si>
     <t>19:23</t>
   </si>
   <si>
     <t>53;7</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub72</t>
-  </si>
-  <si>
     <t>19:36</t>
   </si>
   <si>
     <t>9;68</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub73</t>
-  </si>
-  <si>
     <t>21:00</t>
   </si>
   <si>
@@ -6041,30 +5876,18 @@
     <t>68;46</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub74</t>
-  </si>
-  <si>
     <t>21:40</t>
   </si>
   <si>
     <t>90;98</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub75</t>
-  </si>
-  <si>
-    <t>Arguedas vs Chanhas sub76</t>
-  </si>
-  <si>
     <t>21:52</t>
   </si>
   <si>
     <t>13;39</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub77</t>
-  </si>
-  <si>
     <t>24:31</t>
   </si>
   <si>
@@ -6074,27 +5897,18 @@
     <t>12;44</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub78</t>
-  </si>
-  <si>
     <t>24:38</t>
   </si>
   <si>
     <t>20;41</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub79</t>
-  </si>
-  <si>
     <t>24:57</t>
   </si>
   <si>
     <t>44;51</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub80</t>
-  </si>
-  <si>
     <t>25:25</t>
   </si>
   <si>
@@ -6104,27 +5918,18 @@
     <t>93;99 92;54</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub81</t>
-  </si>
-  <si>
     <t>25:33</t>
   </si>
   <si>
     <t>84;53</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub82</t>
-  </si>
-  <si>
     <t>25:32</t>
   </si>
   <si>
     <t>67;40</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub83</t>
-  </si>
-  <si>
     <t>25:37</t>
   </si>
   <si>
@@ -6134,9 +5939,6 @@
     <t>49;49</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub84</t>
-  </si>
-  <si>
     <t>26:11</t>
   </si>
   <si>
@@ -6146,18 +5948,12 @@
     <t>47;11</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub85</t>
-  </si>
-  <si>
     <t>26:48</t>
   </si>
   <si>
     <t>9;74</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub86</t>
-  </si>
-  <si>
     <t>27:29</t>
   </si>
   <si>
@@ -6167,27 +5963,18 @@
     <t>43;66</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub87</t>
-  </si>
-  <si>
     <t>27:44</t>
   </si>
   <si>
     <t>22;41</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub88</t>
-  </si>
-  <si>
     <t>28:07</t>
   </si>
   <si>
     <t>34;8</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub89</t>
-  </si>
-  <si>
     <t>28:28</t>
   </si>
   <si>
@@ -6197,24 +5984,15 @@
     <t>1;2 7;49</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub90</t>
-  </si>
-  <si>
     <t>28:41</t>
   </si>
   <si>
     <t>28;33</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub91</t>
-  </si>
-  <si>
     <t>94;1 96;36</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub92</t>
-  </si>
-  <si>
     <t>29:19</t>
   </si>
   <si>
@@ -6224,84 +6002,54 @@
     <t>80;1 91;16</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub93</t>
-  </si>
-  <si>
     <t>29:51</t>
   </si>
   <si>
     <t>94;58</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub94</t>
-  </si>
-  <si>
     <t>30:59</t>
   </si>
   <si>
     <t>4;57 8;68</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub95</t>
-  </si>
-  <si>
     <t>32:09</t>
   </si>
   <si>
     <t>19;38</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub96</t>
-  </si>
-  <si>
     <t>32:07</t>
   </si>
   <si>
     <t>51;44</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub97</t>
-  </si>
-  <si>
     <t>32:47</t>
   </si>
   <si>
     <t>52;39</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub98</t>
-  </si>
-  <si>
     <t>10;44</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub99</t>
-  </si>
-  <si>
     <t>33:22</t>
   </si>
   <si>
     <t>34;33 30;65</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub100</t>
-  </si>
-  <si>
     <t>33:56</t>
   </si>
   <si>
     <t>37;96</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub101</t>
-  </si>
-  <si>
     <t>94;57</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub102</t>
-  </si>
-  <si>
     <t>34:37</t>
   </si>
   <si>
@@ -6311,18 +6059,12 @@
     <t>73;87</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub103</t>
-  </si>
-  <si>
     <t>35:22</t>
   </si>
   <si>
     <t>99;100 95;55</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub104</t>
-  </si>
-  <si>
     <t>CAMBIO</t>
   </si>
   <si>
@@ -6332,18 +6074,12 @@
     <t>35:47</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub105</t>
-  </si>
-  <si>
     <t>36:02</t>
   </si>
   <si>
     <t>94;41</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub106</t>
-  </si>
-  <si>
     <t>37:39</t>
   </si>
   <si>
@@ -6356,9 +6092,6 @@
     <t>35;28</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub107</t>
-  </si>
-  <si>
     <t>38:18</t>
   </si>
   <si>
@@ -6368,9 +6101,6 @@
     <t>27;89</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub108</t>
-  </si>
-  <si>
     <t>39:08</t>
   </si>
   <si>
@@ -6380,9 +6110,6 @@
     <t>8;91</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub109</t>
-  </si>
-  <si>
     <t>39:34</t>
   </si>
   <si>
@@ -6392,9 +6119,6 @@
     <t>49;54 57;37</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub110</t>
-  </si>
-  <si>
     <t>39:58</t>
   </si>
   <si>
@@ -6404,9 +6128,6 @@
     <t>21;13</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub111</t>
-  </si>
-  <si>
     <t>40:12</t>
   </si>
   <si>
@@ -6419,9 +6140,6 @@
     <t>Perdida</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub112</t>
-  </si>
-  <si>
     <t>40:57</t>
   </si>
   <si>
@@ -6431,18 +6149,12 @@
     <t>38;64</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub113</t>
-  </si>
-  <si>
     <t>41:48</t>
   </si>
   <si>
     <t>92;16</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub114</t>
-  </si>
-  <si>
     <t>42:27</t>
   </si>
   <si>
@@ -6452,9 +6164,6 @@
     <t>94;38</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub115</t>
-  </si>
-  <si>
     <t>42:37</t>
   </si>
   <si>
@@ -6464,9 +6173,6 @@
     <t>3;9</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub116</t>
-  </si>
-  <si>
     <t>43:33</t>
   </si>
   <si>
@@ -6476,9 +6182,6 @@
     <t>42;58</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub117</t>
-  </si>
-  <si>
     <t>43:37</t>
   </si>
   <si>
@@ -6488,9 +6191,6 @@
     <t>45;60</t>
   </si>
   <si>
-    <t>Arguedas vs Chanhas sub118</t>
-  </si>
-  <si>
     <t>FIN 1T</t>
   </si>
   <si>
@@ -6498,9 +6198,6 @@
   </si>
   <si>
     <t>44:01</t>
-  </si>
-  <si>
-    <t>Arguedas vs Chanhas sub119</t>
   </si>
 </sst>
 </file>
@@ -7352,7 +7049,7 @@
     <col customWidth="1" min="5" max="5" width="10.63"/>
     <col customWidth="1" min="6" max="6" width="17.88"/>
     <col customWidth="1" min="7" max="7" width="17.25"/>
-    <col customWidth="1" min="8" max="8" width="16.88"/>
+    <col customWidth="1" min="8" max="8" width="24.63"/>
     <col customWidth="1" min="9" max="9" width="30.25"/>
     <col customWidth="1" min="10" max="11" width="16.88"/>
     <col customWidth="1" min="12" max="12" width="13.25"/>
@@ -31473,7 +31170,7 @@
         <v>1455</v>
       </c>
       <c r="H603" s="7" t="s">
-        <v>1841</v>
+        <v>1836</v>
       </c>
       <c r="I603" s="8" t="s">
         <v>1837</v>
@@ -31505,14 +31202,14 @@
         <v>73</v>
       </c>
       <c r="E604" s="36" t="s">
-        <v>1842</v>
+        <v>1841</v>
       </c>
       <c r="F604" s="25"/>
       <c r="G604" s="36" t="s">
         <v>1147</v>
       </c>
       <c r="H604" s="7" t="s">
-        <v>1843</v>
+        <v>1836</v>
       </c>
       <c r="I604" s="8" t="s">
         <v>1837</v>
@@ -31541,17 +31238,17 @@
         <v>1456</v>
       </c>
       <c r="D605" s="69" t="s">
-        <v>1844</v>
+        <v>1842</v>
       </c>
       <c r="E605" s="37" t="s">
-        <v>1845</v>
+        <v>1843</v>
       </c>
       <c r="F605" s="37" t="s">
         <v>1095</v>
       </c>
       <c r="G605" s="30"/>
       <c r="H605" s="7" t="s">
-        <v>1846</v>
+        <v>1836</v>
       </c>
       <c r="I605" s="8" t="s">
         <v>1837</v>
@@ -31583,7 +31280,7 @@
         <v>80</v>
       </c>
       <c r="E606" s="36" t="s">
-        <v>1845</v>
+        <v>1843</v>
       </c>
       <c r="F606" s="36" t="s">
         <v>1840</v>
@@ -31592,7 +31289,7 @@
         <v>1111</v>
       </c>
       <c r="H606" s="7" t="s">
-        <v>1847</v>
+        <v>1836</v>
       </c>
       <c r="I606" s="8" t="s">
         <v>1837</v>
@@ -31615,16 +31312,16 @@
         <v>1148</v>
       </c>
       <c r="B607" s="69" t="s">
-        <v>1848</v>
+        <v>1844</v>
       </c>
       <c r="C607" s="69" t="s">
-        <v>1848</v>
+        <v>1844</v>
       </c>
       <c r="D607" s="69" t="s">
         <v>114</v>
       </c>
       <c r="E607" s="37" t="s">
-        <v>1849</v>
+        <v>1845</v>
       </c>
       <c r="F607" s="37" t="s">
         <v>1164</v>
@@ -31633,7 +31330,7 @@
         <v>1164</v>
       </c>
       <c r="H607" s="7" t="s">
-        <v>1850</v>
+        <v>1836</v>
       </c>
       <c r="I607" s="8" t="s">
         <v>1837</v>
@@ -31665,7 +31362,7 @@
         <v>130</v>
       </c>
       <c r="E608" s="36" t="s">
-        <v>1851</v>
+        <v>1846</v>
       </c>
       <c r="F608" s="36" t="s">
         <v>1840</v>
@@ -31674,7 +31371,7 @@
         <v>1123</v>
       </c>
       <c r="H608" s="7" t="s">
-        <v>1852</v>
+        <v>1836</v>
       </c>
       <c r="I608" s="8" t="s">
         <v>1837</v>
@@ -31706,7 +31403,7 @@
         <v>135</v>
       </c>
       <c r="E609" s="37" t="s">
-        <v>1853</v>
+        <v>1847</v>
       </c>
       <c r="F609" s="37" t="s">
         <v>1116</v>
@@ -31715,7 +31412,7 @@
         <v>1087</v>
       </c>
       <c r="H609" s="7" t="s">
-        <v>1854</v>
+        <v>1836</v>
       </c>
       <c r="I609" s="8" t="s">
         <v>1837</v>
@@ -31738,23 +31435,23 @@
         <v>1083</v>
       </c>
       <c r="B610" s="64" t="s">
-        <v>1855</v>
+        <v>1848</v>
       </c>
       <c r="C610" s="64" t="s">
-        <v>1855</v>
+        <v>1848</v>
       </c>
       <c r="D610" s="64" t="s">
         <v>147</v>
       </c>
       <c r="E610" s="36" t="s">
-        <v>1856</v>
+        <v>1849</v>
       </c>
       <c r="F610" s="36" t="s">
         <v>1116</v>
       </c>
       <c r="G610" s="25"/>
       <c r="H610" s="7" t="s">
-        <v>1857</v>
+        <v>1836</v>
       </c>
       <c r="I610" s="8" t="s">
         <v>1837</v>
@@ -31777,23 +31474,23 @@
         <v>1112</v>
       </c>
       <c r="B611" s="69" t="s">
-        <v>1858</v>
+        <v>1850</v>
       </c>
       <c r="C611" s="69" t="s">
-        <v>1858</v>
+        <v>1850</v>
       </c>
       <c r="D611" s="69" t="s">
-        <v>1859</v>
+        <v>1851</v>
       </c>
       <c r="E611" s="37" t="s">
-        <v>1860</v>
+        <v>1852</v>
       </c>
       <c r="F611" s="37" t="s">
         <v>1116</v>
       </c>
       <c r="G611" s="30"/>
       <c r="H611" s="7" t="s">
-        <v>1861</v>
+        <v>1836</v>
       </c>
       <c r="I611" s="8" t="s">
         <v>1837</v>
@@ -31816,23 +31513,23 @@
         <v>1148</v>
       </c>
       <c r="B612" s="64" t="s">
-        <v>1862</v>
+        <v>1853</v>
       </c>
       <c r="C612" s="64" t="s">
-        <v>1862</v>
+        <v>1853</v>
       </c>
       <c r="D612" s="64" t="s">
-        <v>1863</v>
+        <v>1854</v>
       </c>
       <c r="E612" s="36" t="s">
-        <v>1864</v>
+        <v>1855</v>
       </c>
       <c r="F612" s="25"/>
       <c r="G612" s="36" t="s">
         <v>1111</v>
       </c>
       <c r="H612" s="7" t="s">
-        <v>1865</v>
+        <v>1836</v>
       </c>
       <c r="I612" s="8" t="s">
         <v>1837</v>
@@ -31861,19 +31558,19 @@
         <v>184</v>
       </c>
       <c r="D613" s="69" t="s">
-        <v>1866</v>
+        <v>1856</v>
       </c>
       <c r="E613" s="37" t="s">
-        <v>1867</v>
+        <v>1857</v>
       </c>
       <c r="F613" s="37" t="s">
         <v>1840</v>
       </c>
       <c r="G613" s="37" t="s">
-        <v>1868</v>
+        <v>1858</v>
       </c>
       <c r="H613" s="7" t="s">
-        <v>1869</v>
+        <v>1836</v>
       </c>
       <c r="I613" s="8" t="s">
         <v>1837</v>
@@ -31902,10 +31599,10 @@
         <v>195</v>
       </c>
       <c r="D614" s="64" t="s">
-        <v>1870</v>
+        <v>1859</v>
       </c>
       <c r="E614" s="36" t="s">
-        <v>1871</v>
+        <v>1860</v>
       </c>
       <c r="F614" s="36" t="s">
         <v>1127</v>
@@ -31914,7 +31611,7 @@
         <v>1147</v>
       </c>
       <c r="H614" s="7" t="s">
-        <v>1872</v>
+        <v>1836</v>
       </c>
       <c r="I614" s="8" t="s">
         <v>1837</v>
@@ -31943,10 +31640,10 @@
         <v>197</v>
       </c>
       <c r="D615" s="69" t="s">
-        <v>1873</v>
+        <v>1861</v>
       </c>
       <c r="E615" s="37" t="s">
-        <v>1874</v>
+        <v>1862</v>
       </c>
       <c r="F615" s="37" t="s">
         <v>1441</v>
@@ -31955,7 +31652,7 @@
         <v>1111</v>
       </c>
       <c r="H615" s="7" t="s">
-        <v>1875</v>
+        <v>1836</v>
       </c>
       <c r="I615" s="8" t="s">
         <v>1837</v>
@@ -31978,16 +31675,16 @@
         <v>1088</v>
       </c>
       <c r="B616" s="64" t="s">
-        <v>1876</v>
+        <v>1863</v>
       </c>
       <c r="C616" s="64" t="s">
-        <v>1876</v>
+        <v>1863</v>
       </c>
       <c r="D616" s="64" t="s">
         <v>201</v>
       </c>
       <c r="E616" s="36" t="s">
-        <v>1877</v>
+        <v>1864</v>
       </c>
       <c r="F616" s="36" t="s">
         <v>1127</v>
@@ -31996,7 +31693,7 @@
         <v>1455</v>
       </c>
       <c r="H616" s="7" t="s">
-        <v>1878</v>
+        <v>1836</v>
       </c>
       <c r="I616" s="8" t="s">
         <v>1837</v>
@@ -32019,25 +31716,25 @@
         <v>1107</v>
       </c>
       <c r="B617" s="69" t="s">
-        <v>1879</v>
+        <v>1865</v>
       </c>
       <c r="C617" s="69" t="s">
-        <v>1879</v>
+        <v>1865</v>
       </c>
       <c r="D617" s="69" t="s">
         <v>1485</v>
       </c>
       <c r="E617" s="37" t="s">
-        <v>1880</v>
+        <v>1866</v>
       </c>
       <c r="F617" s="37" t="s">
-        <v>1881</v>
+        <v>1867</v>
       </c>
       <c r="G617" s="37" t="s">
         <v>1123</v>
       </c>
       <c r="H617" s="7" t="s">
-        <v>1882</v>
+        <v>1836</v>
       </c>
       <c r="I617" s="8" t="s">
         <v>1837</v>
@@ -32069,14 +31766,14 @@
         <v>226</v>
       </c>
       <c r="E618" s="36" t="s">
-        <v>1883</v>
+        <v>1868</v>
       </c>
       <c r="F618" s="36" t="s">
         <v>1116</v>
       </c>
       <c r="G618" s="25"/>
       <c r="H618" s="7" t="s">
-        <v>1884</v>
+        <v>1836</v>
       </c>
       <c r="I618" s="8" t="s">
         <v>1837</v>
@@ -32108,7 +31805,7 @@
         <v>246</v>
       </c>
       <c r="E619" s="37" t="s">
-        <v>1885</v>
+        <v>1869</v>
       </c>
       <c r="F619" s="37" t="s">
         <v>1441</v>
@@ -32117,7 +31814,7 @@
         <v>1123</v>
       </c>
       <c r="H619" s="7" t="s">
-        <v>1886</v>
+        <v>1836</v>
       </c>
       <c r="I619" s="8" t="s">
         <v>1837</v>
@@ -32146,17 +31843,17 @@
         <v>251</v>
       </c>
       <c r="D620" s="64" t="s">
-        <v>1887</v>
+        <v>1870</v>
       </c>
       <c r="E620" s="36" t="s">
-        <v>1888</v>
+        <v>1871</v>
       </c>
       <c r="F620" s="25"/>
       <c r="G620" s="36" t="s">
         <v>1147</v>
       </c>
       <c r="H620" s="7" t="s">
-        <v>1889</v>
+        <v>1836</v>
       </c>
       <c r="I620" s="8" t="s">
         <v>1837</v>
@@ -32179,16 +31876,16 @@
         <v>1107</v>
       </c>
       <c r="B621" s="69" t="s">
-        <v>1890</v>
+        <v>1872</v>
       </c>
       <c r="C621" s="69" t="s">
-        <v>1890</v>
+        <v>1872</v>
       </c>
       <c r="D621" s="69" t="s">
-        <v>1891</v>
+        <v>1873</v>
       </c>
       <c r="E621" s="37" t="s">
-        <v>1892</v>
+        <v>1874</v>
       </c>
       <c r="F621" s="37" t="s">
         <v>1840</v>
@@ -32197,7 +31894,7 @@
         <v>1455</v>
       </c>
       <c r="H621" s="7" t="s">
-        <v>1893</v>
+        <v>1836</v>
       </c>
       <c r="I621" s="8" t="s">
         <v>1837</v>
@@ -32220,23 +31917,23 @@
         <v>1083</v>
       </c>
       <c r="B622" s="64" t="s">
-        <v>1894</v>
+        <v>1875</v>
       </c>
       <c r="C622" s="64" t="s">
-        <v>1894</v>
+        <v>1875</v>
       </c>
       <c r="D622" s="64" t="s">
         <v>1490</v>
       </c>
       <c r="E622" s="36" t="s">
-        <v>1895</v>
+        <v>1876</v>
       </c>
       <c r="F622" s="36" t="s">
         <v>1095</v>
       </c>
       <c r="G622" s="25"/>
       <c r="H622" s="7" t="s">
-        <v>1896</v>
+        <v>1836</v>
       </c>
       <c r="I622" s="8" t="s">
         <v>1837</v>
@@ -32265,10 +31962,10 @@
         <v>1490</v>
       </c>
       <c r="D623" s="69" t="s">
-        <v>1897</v>
+        <v>1877</v>
       </c>
       <c r="E623" s="37" t="s">
-        <v>1898</v>
+        <v>1878</v>
       </c>
       <c r="F623" s="37" t="s">
         <v>1840</v>
@@ -32277,7 +31974,7 @@
         <v>1087</v>
       </c>
       <c r="H623" s="7" t="s">
-        <v>1899</v>
+        <v>1836</v>
       </c>
       <c r="I623" s="8" t="s">
         <v>1837</v>
@@ -32309,14 +32006,14 @@
         <v>299</v>
       </c>
       <c r="E624" s="36" t="s">
-        <v>1900</v>
+        <v>1879</v>
       </c>
       <c r="F624" s="25"/>
       <c r="G624" s="36" t="s">
         <v>1147</v>
       </c>
       <c r="H624" s="7" t="s">
-        <v>1901</v>
+        <v>1836</v>
       </c>
       <c r="I624" s="8" t="s">
         <v>1837</v>
@@ -32339,23 +32036,23 @@
         <v>1083</v>
       </c>
       <c r="B625" s="69" t="s">
-        <v>1902</v>
+        <v>1880</v>
       </c>
       <c r="C625" s="69" t="s">
-        <v>1902</v>
+        <v>1880</v>
       </c>
       <c r="D625" s="69" t="s">
-        <v>1903</v>
+        <v>1881</v>
       </c>
       <c r="E625" s="37" t="s">
-        <v>1904</v>
+        <v>1882</v>
       </c>
       <c r="F625" s="37" t="s">
         <v>1116</v>
       </c>
       <c r="G625" s="30"/>
       <c r="H625" s="7" t="s">
-        <v>1905</v>
+        <v>1836</v>
       </c>
       <c r="I625" s="8" t="s">
         <v>1837</v>
@@ -32387,14 +32084,14 @@
         <v>320</v>
       </c>
       <c r="E626" s="36" t="s">
-        <v>1906</v>
+        <v>1883</v>
       </c>
       <c r="F626" s="36" t="s">
         <v>1116</v>
       </c>
       <c r="G626" s="25"/>
       <c r="H626" s="7" t="s">
-        <v>1907</v>
+        <v>1836</v>
       </c>
       <c r="I626" s="8" t="s">
         <v>1837</v>
@@ -32417,23 +32114,23 @@
         <v>1088</v>
       </c>
       <c r="B627" s="69" t="s">
-        <v>1908</v>
+        <v>1884</v>
       </c>
       <c r="C627" s="69" t="s">
-        <v>1908</v>
+        <v>1884</v>
       </c>
       <c r="D627" s="69" t="s">
         <v>330</v>
       </c>
       <c r="E627" s="37" t="s">
-        <v>1909</v>
+        <v>1885</v>
       </c>
       <c r="F627" s="30"/>
       <c r="G627" s="37" t="s">
         <v>1455</v>
       </c>
       <c r="H627" s="7" t="s">
-        <v>1910</v>
+        <v>1836</v>
       </c>
       <c r="I627" s="8" t="s">
         <v>1837</v>
@@ -32456,16 +32153,16 @@
         <v>1107</v>
       </c>
       <c r="B628" s="64" t="s">
-        <v>1911</v>
+        <v>1886</v>
       </c>
       <c r="C628" s="64" t="s">
-        <v>1911</v>
+        <v>1886</v>
       </c>
       <c r="D628" s="64" t="s">
-        <v>1912</v>
+        <v>1887</v>
       </c>
       <c r="E628" s="36" t="s">
-        <v>1913</v>
+        <v>1888</v>
       </c>
       <c r="F628" s="36" t="s">
         <v>1840</v>
@@ -32474,7 +32171,7 @@
         <v>1111</v>
       </c>
       <c r="H628" s="7" t="s">
-        <v>1914</v>
+        <v>1836</v>
       </c>
       <c r="I628" s="8" t="s">
         <v>1837</v>
@@ -32497,16 +32194,16 @@
         <v>1088</v>
       </c>
       <c r="B629" s="69" t="s">
-        <v>1915</v>
+        <v>1889</v>
       </c>
       <c r="C629" s="69" t="s">
-        <v>1915</v>
+        <v>1889</v>
       </c>
       <c r="D629" s="69" t="s">
-        <v>1916</v>
+        <v>1890</v>
       </c>
       <c r="E629" s="37" t="s">
-        <v>1917</v>
+        <v>1891</v>
       </c>
       <c r="F629" s="37" t="s">
         <v>1127</v>
@@ -32515,7 +32212,7 @@
         <v>1147</v>
       </c>
       <c r="H629" s="7" t="s">
-        <v>1918</v>
+        <v>1836</v>
       </c>
       <c r="I629" s="8" t="s">
         <v>1837</v>
@@ -32538,16 +32235,16 @@
         <v>1107</v>
       </c>
       <c r="B630" s="64" t="s">
-        <v>1919</v>
+        <v>1892</v>
       </c>
       <c r="C630" s="64" t="s">
-        <v>1919</v>
+        <v>1892</v>
       </c>
       <c r="D630" s="64" t="s">
         <v>354</v>
       </c>
       <c r="E630" s="36" t="s">
-        <v>1920</v>
+        <v>1893</v>
       </c>
       <c r="F630" s="36" t="s">
         <v>1840</v>
@@ -32556,7 +32253,7 @@
         <v>1111</v>
       </c>
       <c r="H630" s="7" t="s">
-        <v>1921</v>
+        <v>1836</v>
       </c>
       <c r="I630" s="8" t="s">
         <v>1837</v>
@@ -32585,10 +32282,10 @@
         <v>361</v>
       </c>
       <c r="D631" s="69" t="s">
-        <v>1922</v>
+        <v>1894</v>
       </c>
       <c r="E631" s="37" t="s">
-        <v>1923</v>
+        <v>1895</v>
       </c>
       <c r="F631" s="37" t="s">
         <v>1127</v>
@@ -32597,7 +32294,7 @@
         <v>1147</v>
       </c>
       <c r="H631" s="7" t="s">
-        <v>1924</v>
+        <v>1836</v>
       </c>
       <c r="I631" s="8" t="s">
         <v>1837</v>
@@ -32620,16 +32317,16 @@
         <v>1107</v>
       </c>
       <c r="B632" s="64" t="s">
-        <v>1925</v>
+        <v>1896</v>
       </c>
       <c r="C632" s="64" t="s">
-        <v>1926</v>
+        <v>1897</v>
       </c>
       <c r="D632" s="64" t="s">
-        <v>1926</v>
+        <v>1897</v>
       </c>
       <c r="E632" s="36" t="s">
-        <v>1927</v>
+        <v>1898</v>
       </c>
       <c r="F632" s="36" t="s">
         <v>1840</v>
@@ -32638,7 +32335,7 @@
         <v>1123</v>
       </c>
       <c r="H632" s="7" t="s">
-        <v>1928</v>
+        <v>1836</v>
       </c>
       <c r="I632" s="8" t="s">
         <v>1837</v>
@@ -32661,16 +32358,16 @@
         <v>1088</v>
       </c>
       <c r="B633" s="69" t="s">
-        <v>1929</v>
+        <v>1899</v>
       </c>
       <c r="C633" s="69" t="s">
-        <v>1929</v>
+        <v>1899</v>
       </c>
       <c r="D633" s="69" t="s">
         <v>1747</v>
       </c>
       <c r="E633" s="37" t="s">
-        <v>1930</v>
+        <v>1900</v>
       </c>
       <c r="F633" s="37" t="s">
         <v>1127</v>
@@ -32679,7 +32376,7 @@
         <v>1147</v>
       </c>
       <c r="H633" s="7" t="s">
-        <v>1931</v>
+        <v>1836</v>
       </c>
       <c r="I633" s="8" t="s">
         <v>1837</v>
@@ -32711,7 +32408,7 @@
         <v>1749</v>
       </c>
       <c r="E634" s="36" t="s">
-        <v>1932</v>
+        <v>1901</v>
       </c>
       <c r="F634" s="36" t="s">
         <v>1441</v>
@@ -32720,7 +32417,7 @@
         <v>1111</v>
       </c>
       <c r="H634" s="7" t="s">
-        <v>1933</v>
+        <v>1836</v>
       </c>
       <c r="I634" s="8" t="s">
         <v>1837</v>
@@ -32752,14 +32449,14 @@
         <v>391</v>
       </c>
       <c r="E635" s="37" t="s">
-        <v>1934</v>
+        <v>1902</v>
       </c>
       <c r="F635" s="30"/>
       <c r="G635" s="37" t="s">
         <v>1147</v>
       </c>
       <c r="H635" s="7" t="s">
-        <v>1935</v>
+        <v>1836</v>
       </c>
       <c r="I635" s="8" t="s">
         <v>1837</v>
@@ -32788,10 +32485,10 @@
         <v>394</v>
       </c>
       <c r="D636" s="64" t="s">
-        <v>1936</v>
+        <v>1903</v>
       </c>
       <c r="E636" s="36" t="s">
-        <v>1937</v>
+        <v>1904</v>
       </c>
       <c r="F636" s="36" t="s">
         <v>1441</v>
@@ -32800,7 +32497,7 @@
         <v>1164</v>
       </c>
       <c r="H636" s="7" t="s">
-        <v>1938</v>
+        <v>1836</v>
       </c>
       <c r="I636" s="8" t="s">
         <v>1837</v>
@@ -32823,16 +32520,16 @@
         <v>1107</v>
       </c>
       <c r="B637" s="69" t="s">
-        <v>1939</v>
+        <v>1905</v>
       </c>
       <c r="C637" s="69" t="s">
-        <v>1939</v>
+        <v>1905</v>
       </c>
       <c r="D637" s="69" t="s">
         <v>415</v>
       </c>
       <c r="E637" s="37" t="s">
-        <v>1940</v>
+        <v>1906</v>
       </c>
       <c r="F637" s="37" t="s">
         <v>1840</v>
@@ -32841,7 +32538,7 @@
         <v>1087</v>
       </c>
       <c r="H637" s="7" t="s">
-        <v>1941</v>
+        <v>1836</v>
       </c>
       <c r="I637" s="8" t="s">
         <v>1837</v>
@@ -32864,23 +32561,23 @@
         <v>1077</v>
       </c>
       <c r="B638" s="64" t="s">
-        <v>1942</v>
+        <v>1907</v>
       </c>
       <c r="C638" s="64" t="s">
-        <v>1942</v>
+        <v>1907</v>
       </c>
       <c r="D638" s="64" t="s">
         <v>1516</v>
       </c>
       <c r="E638" s="36" t="s">
-        <v>1943</v>
+        <v>1908</v>
       </c>
       <c r="F638" s="25"/>
       <c r="G638" s="36" t="s">
         <v>1082</v>
       </c>
       <c r="H638" s="7" t="s">
-        <v>1944</v>
+        <v>1836</v>
       </c>
       <c r="I638" s="8" t="s">
         <v>1837</v>
@@ -32903,16 +32600,16 @@
         <v>1107</v>
       </c>
       <c r="B639" s="69" t="s">
-        <v>1945</v>
+        <v>1909</v>
       </c>
       <c r="C639" s="69" t="s">
-        <v>1945</v>
+        <v>1909</v>
       </c>
       <c r="D639" s="69" t="s">
-        <v>1946</v>
+        <v>1910</v>
       </c>
       <c r="E639" s="37" t="s">
-        <v>1947</v>
+        <v>1911</v>
       </c>
       <c r="F639" s="37" t="s">
         <v>1217</v>
@@ -32921,7 +32618,7 @@
         <v>1123</v>
       </c>
       <c r="H639" s="7" t="s">
-        <v>1948</v>
+        <v>1836</v>
       </c>
       <c r="I639" s="8" t="s">
         <v>1837</v>
@@ -32953,7 +32650,7 @@
         <v>481</v>
       </c>
       <c r="E640" s="36" t="s">
-        <v>1949</v>
+        <v>1912</v>
       </c>
       <c r="F640" s="36" t="s">
         <v>1086</v>
@@ -32962,7 +32659,7 @@
         <v>1087</v>
       </c>
       <c r="H640" s="7" t="s">
-        <v>1950</v>
+        <v>1836</v>
       </c>
       <c r="I640" s="8" t="s">
         <v>1837</v>
@@ -32985,23 +32682,23 @@
         <v>1077</v>
       </c>
       <c r="B641" s="69" t="s">
-        <v>1951</v>
+        <v>1913</v>
       </c>
       <c r="C641" s="69" t="s">
-        <v>1951</v>
+        <v>1913</v>
       </c>
       <c r="D641" s="69" t="s">
         <v>509</v>
       </c>
       <c r="E641" s="37" t="s">
-        <v>1952</v>
+        <v>1914</v>
       </c>
       <c r="F641" s="30"/>
       <c r="G641" s="37" t="s">
         <v>1455</v>
       </c>
       <c r="H641" s="7" t="s">
-        <v>1953</v>
+        <v>1836</v>
       </c>
       <c r="I641" s="8" t="s">
         <v>1837</v>
@@ -33024,23 +32721,23 @@
         <v>1083</v>
       </c>
       <c r="B642" s="64" t="s">
-        <v>1954</v>
+        <v>1915</v>
       </c>
       <c r="C642" s="64" t="s">
-        <v>1954</v>
+        <v>1915</v>
       </c>
       <c r="D642" s="64" t="s">
         <v>1534</v>
       </c>
       <c r="E642" s="36" t="s">
-        <v>1955</v>
+        <v>1916</v>
       </c>
       <c r="F642" s="36" t="s">
         <v>1116</v>
       </c>
       <c r="G642" s="25"/>
       <c r="H642" s="7" t="s">
-        <v>1956</v>
+        <v>1836</v>
       </c>
       <c r="I642" s="8" t="s">
         <v>1837</v>
@@ -33063,16 +32760,16 @@
         <v>1088</v>
       </c>
       <c r="B643" s="69" t="s">
-        <v>1957</v>
+        <v>1917</v>
       </c>
       <c r="C643" s="69" t="s">
-        <v>1957</v>
+        <v>1917</v>
       </c>
       <c r="D643" s="69" t="s">
-        <v>1958</v>
+        <v>1918</v>
       </c>
       <c r="E643" s="37" t="s">
-        <v>1959</v>
+        <v>1919</v>
       </c>
       <c r="F643" s="37" t="s">
         <v>1127</v>
@@ -33081,7 +32778,7 @@
         <v>1147</v>
       </c>
       <c r="H643" s="7" t="s">
-        <v>1960</v>
+        <v>1836</v>
       </c>
       <c r="I643" s="8" t="s">
         <v>1837</v>
@@ -33104,16 +32801,16 @@
         <v>1148</v>
       </c>
       <c r="B644" s="64" t="s">
-        <v>1961</v>
+        <v>1920</v>
       </c>
       <c r="C644" s="64" t="s">
-        <v>1962</v>
+        <v>1921</v>
       </c>
       <c r="D644" s="64" t="s">
-        <v>1963</v>
+        <v>1922</v>
       </c>
       <c r="E644" s="36" t="s">
-        <v>1964</v>
+        <v>1923</v>
       </c>
       <c r="F644" s="36" t="s">
         <v>1441</v>
@@ -33122,7 +32819,7 @@
         <v>1087</v>
       </c>
       <c r="H644" s="7" t="s">
-        <v>1965</v>
+        <v>1836</v>
       </c>
       <c r="I644" s="8" t="s">
         <v>1837</v>
@@ -33151,10 +32848,10 @@
         <v>1537</v>
       </c>
       <c r="D645" s="69" t="s">
-        <v>1966</v>
+        <v>1924</v>
       </c>
       <c r="E645" s="37" t="s">
-        <v>1967</v>
+        <v>1925</v>
       </c>
       <c r="F645" s="37" t="s">
         <v>1127</v>
@@ -33163,7 +32860,7 @@
         <v>1455</v>
       </c>
       <c r="H645" s="7" t="s">
-        <v>1968</v>
+        <v>1836</v>
       </c>
       <c r="I645" s="8" t="s">
         <v>1837</v>
@@ -33186,23 +32883,23 @@
         <v>1112</v>
       </c>
       <c r="B646" s="64" t="s">
-        <v>1969</v>
+        <v>1926</v>
       </c>
       <c r="C646" s="64" t="s">
-        <v>1969</v>
+        <v>1926</v>
       </c>
       <c r="D646" s="64" t="s">
-        <v>1970</v>
+        <v>1927</v>
       </c>
       <c r="E646" s="36" t="s">
-        <v>1971</v>
+        <v>1928</v>
       </c>
       <c r="F646" s="36" t="s">
         <v>1095</v>
       </c>
       <c r="G646" s="25"/>
       <c r="H646" s="7" t="s">
-        <v>1972</v>
+        <v>1836</v>
       </c>
       <c r="I646" s="8" t="s">
         <v>1837</v>
@@ -33225,16 +32922,16 @@
         <v>1148</v>
       </c>
       <c r="B647" s="69" t="s">
-        <v>1973</v>
+        <v>1929</v>
       </c>
       <c r="C647" s="69" t="s">
-        <v>1973</v>
+        <v>1929</v>
       </c>
       <c r="D647" s="69" t="s">
-        <v>1974</v>
+        <v>1930</v>
       </c>
       <c r="E647" s="37" t="s">
-        <v>1975</v>
+        <v>1931</v>
       </c>
       <c r="F647" s="37" t="s">
         <v>1441</v>
@@ -33243,7 +32940,7 @@
         <v>1111</v>
       </c>
       <c r="H647" s="7" t="s">
-        <v>1976</v>
+        <v>1836</v>
       </c>
       <c r="I647" s="8" t="s">
         <v>1837</v>
@@ -33275,14 +32972,14 @@
         <v>537</v>
       </c>
       <c r="E648" s="36" t="s">
-        <v>1977</v>
+        <v>1932</v>
       </c>
       <c r="F648" s="25"/>
       <c r="G648" s="36" t="s">
         <v>1147</v>
       </c>
       <c r="H648" s="7" t="s">
-        <v>1978</v>
+        <v>1836</v>
       </c>
       <c r="I648" s="8" t="s">
         <v>1837</v>
@@ -33305,16 +33002,16 @@
         <v>1148</v>
       </c>
       <c r="B649" s="69" t="s">
-        <v>1979</v>
+        <v>1933</v>
       </c>
       <c r="C649" s="69" t="s">
-        <v>1979</v>
+        <v>1933</v>
       </c>
       <c r="D649" s="69" t="s">
-        <v>1980</v>
+        <v>1934</v>
       </c>
       <c r="E649" s="37" t="s">
-        <v>1981</v>
+        <v>1935</v>
       </c>
       <c r="F649" s="37" t="s">
         <v>1441</v>
@@ -33323,7 +33020,7 @@
         <v>1087</v>
       </c>
       <c r="H649" s="7" t="s">
-        <v>1982</v>
+        <v>1836</v>
       </c>
       <c r="I649" s="8" t="s">
         <v>1837</v>
@@ -33346,23 +33043,23 @@
         <v>1083</v>
       </c>
       <c r="B650" s="64" t="s">
-        <v>1983</v>
+        <v>1936</v>
       </c>
       <c r="C650" s="64" t="s">
-        <v>1983</v>
+        <v>1936</v>
       </c>
       <c r="D650" s="64" t="s">
         <v>550</v>
       </c>
       <c r="E650" s="36" t="s">
-        <v>1984</v>
+        <v>1937</v>
       </c>
       <c r="F650" s="36" t="s">
         <v>1086</v>
       </c>
       <c r="G650" s="25"/>
       <c r="H650" s="7" t="s">
-        <v>1985</v>
+        <v>1836</v>
       </c>
       <c r="I650" s="8" t="s">
         <v>1837</v>
@@ -33385,23 +33082,23 @@
         <v>1088</v>
       </c>
       <c r="B651" s="69" t="s">
-        <v>1986</v>
+        <v>1938</v>
       </c>
       <c r="C651" s="69" t="s">
-        <v>1986</v>
+        <v>1938</v>
       </c>
       <c r="D651" s="69" t="s">
         <v>550</v>
       </c>
       <c r="E651" s="37" t="s">
-        <v>1987</v>
+        <v>1939</v>
       </c>
       <c r="F651" s="30"/>
       <c r="G651" s="37" t="s">
         <v>1082</v>
       </c>
       <c r="H651" s="7" t="s">
-        <v>1988</v>
+        <v>1836</v>
       </c>
       <c r="I651" s="8" t="s">
         <v>1837</v>
@@ -33433,7 +33130,7 @@
         <v>564</v>
       </c>
       <c r="E652" s="36" t="s">
-        <v>1989</v>
+        <v>1940</v>
       </c>
       <c r="F652" s="36" t="s">
         <v>1840</v>
@@ -33442,7 +33139,7 @@
         <v>1123</v>
       </c>
       <c r="H652" s="7" t="s">
-        <v>1990</v>
+        <v>1836</v>
       </c>
       <c r="I652" s="8" t="s">
         <v>1837</v>
@@ -33474,14 +33171,14 @@
         <v>570</v>
       </c>
       <c r="E653" s="37" t="s">
-        <v>1991</v>
+        <v>1941</v>
       </c>
       <c r="F653" s="37" t="s">
         <v>1116</v>
       </c>
       <c r="G653" s="30"/>
       <c r="H653" s="7" t="s">
-        <v>1992</v>
+        <v>1836</v>
       </c>
       <c r="I653" s="8" t="s">
         <v>1837</v>
@@ -33513,14 +33210,14 @@
         <v>607</v>
       </c>
       <c r="E654" s="36" t="s">
-        <v>1993</v>
+        <v>1942</v>
       </c>
       <c r="F654" s="25"/>
       <c r="G654" s="36" t="s">
         <v>1082</v>
       </c>
       <c r="H654" s="7" t="s">
-        <v>1994</v>
+        <v>1836</v>
       </c>
       <c r="I654" s="8" t="s">
         <v>1837</v>
@@ -33549,10 +33246,10 @@
         <v>605</v>
       </c>
       <c r="D655" s="69" t="s">
-        <v>1995</v>
+        <v>1943</v>
       </c>
       <c r="E655" s="37" t="s">
-        <v>1996</v>
+        <v>1944</v>
       </c>
       <c r="F655" s="37" t="s">
         <v>1840</v>
@@ -33561,7 +33258,7 @@
         <v>1123</v>
       </c>
       <c r="H655" s="7" t="s">
-        <v>1997</v>
+        <v>1836</v>
       </c>
       <c r="I655" s="8" t="s">
         <v>1837</v>
@@ -33590,17 +33287,17 @@
         <v>630</v>
       </c>
       <c r="D656" s="64" t="s">
-        <v>1998</v>
+        <v>1945</v>
       </c>
       <c r="E656" s="36" t="s">
-        <v>1999</v>
+        <v>1946</v>
       </c>
       <c r="F656" s="25"/>
       <c r="G656" s="36" t="s">
         <v>1133</v>
       </c>
       <c r="H656" s="7" t="s">
-        <v>2000</v>
+        <v>1836</v>
       </c>
       <c r="I656" s="8" t="s">
         <v>1837</v>
@@ -33623,16 +33320,16 @@
         <v>1107</v>
       </c>
       <c r="B657" s="69" t="s">
-        <v>2001</v>
+        <v>1947</v>
       </c>
       <c r="C657" s="69" t="s">
-        <v>2001</v>
+        <v>1947</v>
       </c>
       <c r="D657" s="69" t="s">
         <v>670</v>
       </c>
       <c r="E657" s="37" t="s">
-        <v>2002</v>
+        <v>1948</v>
       </c>
       <c r="F657" s="37" t="s">
         <v>1840</v>
@@ -33641,7 +33338,7 @@
         <v>1455</v>
       </c>
       <c r="H657" s="7" t="s">
-        <v>2003</v>
+        <v>1836</v>
       </c>
       <c r="I657" s="8" t="s">
         <v>1837</v>
@@ -33664,16 +33361,16 @@
         <v>1083</v>
       </c>
       <c r="B658" s="64" t="s">
-        <v>2004</v>
+        <v>1949</v>
       </c>
       <c r="C658" s="64" t="s">
-        <v>2004</v>
+        <v>1949</v>
       </c>
       <c r="D658" s="64" t="s">
-        <v>2005</v>
+        <v>1950</v>
       </c>
       <c r="E658" s="36" t="s">
-        <v>2006</v>
+        <v>1951</v>
       </c>
       <c r="F658" s="36" t="s">
         <v>1095</v>
@@ -33682,7 +33379,7 @@
         <v>1087</v>
       </c>
       <c r="H658" s="7" t="s">
-        <v>2007</v>
+        <v>1836</v>
       </c>
       <c r="I658" s="8" t="s">
         <v>1837</v>
@@ -33711,10 +33408,10 @@
         <v>1577</v>
       </c>
       <c r="D659" s="69" t="s">
-        <v>2008</v>
+        <v>1952</v>
       </c>
       <c r="E659" s="37" t="s">
-        <v>2009</v>
+        <v>1953</v>
       </c>
       <c r="F659" s="37" t="s">
         <v>1116</v>
@@ -33723,7 +33420,7 @@
         <v>1123</v>
       </c>
       <c r="H659" s="7" t="s">
-        <v>2010</v>
+        <v>1836</v>
       </c>
       <c r="I659" s="8" t="s">
         <v>1837</v>
@@ -33746,23 +33443,23 @@
         <v>1088</v>
       </c>
       <c r="B660" s="64" t="s">
-        <v>2008</v>
+        <v>1952</v>
       </c>
       <c r="C660" s="64" t="s">
-        <v>2008</v>
+        <v>1952</v>
       </c>
       <c r="D660" s="64" t="s">
         <v>678</v>
       </c>
       <c r="E660" s="36" t="s">
-        <v>1888</v>
+        <v>1871</v>
       </c>
       <c r="F660" s="25"/>
       <c r="G660" s="36" t="s">
         <v>1133</v>
       </c>
       <c r="H660" s="7" t="s">
-        <v>2011</v>
+        <v>1836</v>
       </c>
       <c r="I660" s="8" t="s">
         <v>1837</v>
@@ -33785,16 +33482,16 @@
         <v>1107</v>
       </c>
       <c r="B661" s="69" t="s">
-        <v>2012</v>
+        <v>1954</v>
       </c>
       <c r="C661" s="69" t="s">
-        <v>2012</v>
+        <v>1954</v>
       </c>
       <c r="D661" s="69" t="s">
         <v>695</v>
       </c>
       <c r="E661" s="37" t="s">
-        <v>2013</v>
+        <v>1955</v>
       </c>
       <c r="F661" s="37" t="s">
         <v>1840</v>
@@ -33803,7 +33500,7 @@
         <v>1111</v>
       </c>
       <c r="H661" s="7" t="s">
-        <v>2014</v>
+        <v>1836</v>
       </c>
       <c r="I661" s="8" t="s">
         <v>1837</v>
@@ -33826,16 +33523,16 @@
         <v>1107</v>
       </c>
       <c r="B662" s="64" t="s">
-        <v>2015</v>
+        <v>1956</v>
       </c>
       <c r="C662" s="64" t="s">
-        <v>2015</v>
+        <v>1956</v>
       </c>
       <c r="D662" s="64" t="s">
-        <v>2016</v>
+        <v>1957</v>
       </c>
       <c r="E662" s="36" t="s">
-        <v>2017</v>
+        <v>1958</v>
       </c>
       <c r="F662" s="36" t="s">
         <v>1840</v>
@@ -33844,7 +33541,7 @@
         <v>1455</v>
       </c>
       <c r="H662" s="7" t="s">
-        <v>2018</v>
+        <v>1836</v>
       </c>
       <c r="I662" s="8" t="s">
         <v>1837</v>
@@ -33867,16 +33564,16 @@
         <v>1107</v>
       </c>
       <c r="B663" s="69" t="s">
-        <v>2019</v>
+        <v>1959</v>
       </c>
       <c r="C663" s="69" t="s">
-        <v>2019</v>
+        <v>1959</v>
       </c>
       <c r="D663" s="69" t="s">
         <v>1596</v>
       </c>
       <c r="E663" s="37" t="s">
-        <v>2020</v>
+        <v>1960</v>
       </c>
       <c r="F663" s="37" t="s">
         <v>1840</v>
@@ -33885,7 +33582,7 @@
         <v>1455</v>
       </c>
       <c r="H663" s="7" t="s">
-        <v>2021</v>
+        <v>1836</v>
       </c>
       <c r="I663" s="8" t="s">
         <v>1837</v>
@@ -33908,16 +33605,16 @@
         <v>1107</v>
       </c>
       <c r="B664" s="64" t="s">
-        <v>2022</v>
+        <v>1961</v>
       </c>
       <c r="C664" s="64" t="s">
-        <v>2022</v>
+        <v>1961</v>
       </c>
       <c r="D664" s="64" t="s">
         <v>769</v>
       </c>
       <c r="E664" s="36" t="s">
-        <v>2023</v>
+        <v>1962</v>
       </c>
       <c r="F664" s="36" t="s">
         <v>1840</v>
@@ -33926,7 +33623,7 @@
         <v>1123</v>
       </c>
       <c r="H664" s="7" t="s">
-        <v>2024</v>
+        <v>1836</v>
       </c>
       <c r="I664" s="8" t="s">
         <v>1837</v>
@@ -33949,23 +33646,23 @@
         <v>1083</v>
       </c>
       <c r="B665" s="69" t="s">
-        <v>2025</v>
+        <v>1963</v>
       </c>
       <c r="C665" s="69" t="s">
-        <v>2025</v>
+        <v>1963</v>
       </c>
       <c r="D665" s="69" t="s">
-        <v>2026</v>
+        <v>1964</v>
       </c>
       <c r="E665" s="37" t="s">
-        <v>2027</v>
+        <v>1965</v>
       </c>
       <c r="F665" s="37" t="s">
         <v>1116</v>
       </c>
       <c r="G665" s="30"/>
       <c r="H665" s="7" t="s">
-        <v>2028</v>
+        <v>1836</v>
       </c>
       <c r="I665" s="8" t="s">
         <v>1837</v>
@@ -33994,10 +33691,10 @@
         <v>783</v>
       </c>
       <c r="D666" s="64" t="s">
-        <v>2029</v>
+        <v>1966</v>
       </c>
       <c r="E666" s="36" t="s">
-        <v>2030</v>
+        <v>1967</v>
       </c>
       <c r="F666" s="36" t="s">
         <v>1127</v>
@@ -34006,7 +33703,7 @@
         <v>1147</v>
       </c>
       <c r="H666" s="7" t="s">
-        <v>2031</v>
+        <v>1836</v>
       </c>
       <c r="I666" s="8" t="s">
         <v>1837</v>
@@ -34029,16 +33726,16 @@
         <v>1148</v>
       </c>
       <c r="B667" s="69" t="s">
-        <v>2026</v>
+        <v>1964</v>
       </c>
       <c r="C667" s="69" t="s">
-        <v>2032</v>
+        <v>1968</v>
       </c>
       <c r="D667" s="69" t="s">
         <v>785</v>
       </c>
       <c r="E667" s="37" t="s">
-        <v>2033</v>
+        <v>1969</v>
       </c>
       <c r="F667" s="37" t="s">
         <v>1441</v>
@@ -34047,7 +33744,7 @@
         <v>1455</v>
       </c>
       <c r="H667" s="7" t="s">
-        <v>2034</v>
+        <v>1836</v>
       </c>
       <c r="I667" s="8" t="s">
         <v>1837</v>
@@ -34070,16 +33767,16 @@
         <v>1148</v>
       </c>
       <c r="B668" s="64" t="s">
-        <v>2035</v>
+        <v>1970</v>
       </c>
       <c r="C668" s="64" t="s">
-        <v>2035</v>
+        <v>1970</v>
       </c>
       <c r="D668" s="64" t="s">
-        <v>2036</v>
+        <v>1971</v>
       </c>
       <c r="E668" s="36" t="s">
-        <v>2037</v>
+        <v>1972</v>
       </c>
       <c r="F668" s="36" t="s">
         <v>1164</v>
@@ -34088,7 +33785,7 @@
         <v>1111</v>
       </c>
       <c r="H668" s="7" t="s">
-        <v>2038</v>
+        <v>1836</v>
       </c>
       <c r="I668" s="8" t="s">
         <v>1837</v>
@@ -34111,23 +33808,23 @@
         <v>1112</v>
       </c>
       <c r="B669" s="69" t="s">
-        <v>2039</v>
+        <v>1973</v>
       </c>
       <c r="C669" s="69" t="s">
-        <v>2039</v>
+        <v>1973</v>
       </c>
       <c r="D669" s="69" t="s">
-        <v>2040</v>
+        <v>1974</v>
       </c>
       <c r="E669" s="37" t="s">
-        <v>2041</v>
+        <v>1975</v>
       </c>
       <c r="F669" s="37" t="s">
         <v>1095</v>
       </c>
       <c r="G669" s="30"/>
       <c r="H669" s="7" t="s">
-        <v>2042</v>
+        <v>1836</v>
       </c>
       <c r="I669" s="8" t="s">
         <v>1837</v>
@@ -34156,17 +33853,17 @@
         <v>1608</v>
       </c>
       <c r="D670" s="64" t="s">
-        <v>2043</v>
+        <v>1976</v>
       </c>
       <c r="E670" s="36" t="s">
-        <v>2044</v>
+        <v>1977</v>
       </c>
       <c r="F670" s="25"/>
       <c r="G670" s="36" t="s">
         <v>1147</v>
       </c>
       <c r="H670" s="7" t="s">
-        <v>2045</v>
+        <v>1836</v>
       </c>
       <c r="I670" s="8" t="s">
         <v>1837</v>
@@ -34189,23 +33886,23 @@
         <v>1083</v>
       </c>
       <c r="B671" s="69" t="s">
-        <v>2046</v>
+        <v>1978</v>
       </c>
       <c r="C671" s="69" t="s">
-        <v>2046</v>
+        <v>1978</v>
       </c>
       <c r="D671" s="69" t="s">
-        <v>2047</v>
+        <v>1979</v>
       </c>
       <c r="E671" s="37" t="s">
-        <v>2048</v>
+        <v>1980</v>
       </c>
       <c r="F671" s="37" t="s">
         <v>1095</v>
       </c>
       <c r="G671" s="30"/>
       <c r="H671" s="7" t="s">
-        <v>2049</v>
+        <v>1836</v>
       </c>
       <c r="I671" s="8" t="s">
         <v>1837</v>
@@ -34228,16 +33925,16 @@
         <v>1107</v>
       </c>
       <c r="B672" s="64" t="s">
-        <v>2050</v>
+        <v>1981</v>
       </c>
       <c r="C672" s="64" t="s">
-        <v>2050</v>
+        <v>1981</v>
       </c>
       <c r="D672" s="64" t="s">
         <v>829</v>
       </c>
       <c r="E672" s="36" t="s">
-        <v>2051</v>
+        <v>1982</v>
       </c>
       <c r="F672" s="36" t="s">
         <v>1840</v>
@@ -34246,7 +33943,7 @@
         <v>1111</v>
       </c>
       <c r="H672" s="7" t="s">
-        <v>2052</v>
+        <v>1836</v>
       </c>
       <c r="I672" s="8" t="s">
         <v>1837</v>
@@ -34275,17 +33972,17 @@
         <v>828</v>
       </c>
       <c r="D673" s="69" t="s">
-        <v>2053</v>
+        <v>1983</v>
       </c>
       <c r="E673" s="37" t="s">
-        <v>2054</v>
+        <v>1984</v>
       </c>
       <c r="F673" s="30"/>
       <c r="G673" s="37" t="s">
         <v>1455</v>
       </c>
       <c r="H673" s="7" t="s">
-        <v>2055</v>
+        <v>1836</v>
       </c>
       <c r="I673" s="8" t="s">
         <v>1837</v>
@@ -34308,23 +34005,23 @@
         <v>1112</v>
       </c>
       <c r="B674" s="64" t="s">
-        <v>2056</v>
+        <v>1985</v>
       </c>
       <c r="C674" s="64" t="s">
-        <v>2056</v>
+        <v>1985</v>
       </c>
       <c r="D674" s="64" t="s">
-        <v>2057</v>
+        <v>1986</v>
       </c>
       <c r="E674" s="36" t="s">
-        <v>2058</v>
+        <v>1987</v>
       </c>
       <c r="F674" s="36" t="s">
         <v>1086</v>
       </c>
       <c r="G674" s="25"/>
       <c r="H674" s="7" t="s">
-        <v>2059</v>
+        <v>1836</v>
       </c>
       <c r="I674" s="8" t="s">
         <v>1837</v>
@@ -34347,16 +34044,16 @@
         <v>1148</v>
       </c>
       <c r="B675" s="69" t="s">
-        <v>2060</v>
+        <v>1988</v>
       </c>
       <c r="C675" s="69" t="s">
-        <v>2060</v>
+        <v>1988</v>
       </c>
       <c r="D675" s="69" t="s">
         <v>856</v>
       </c>
       <c r="E675" s="37" t="s">
-        <v>2061</v>
+        <v>1989</v>
       </c>
       <c r="F675" s="37" t="s">
         <v>1441</v>
@@ -34365,7 +34062,7 @@
         <v>1123</v>
       </c>
       <c r="H675" s="7" t="s">
-        <v>2062</v>
+        <v>1836</v>
       </c>
       <c r="I675" s="8" t="s">
         <v>1837</v>
@@ -34397,14 +34094,14 @@
         <v>864</v>
       </c>
       <c r="E676" s="36" t="s">
-        <v>2063</v>
+        <v>1990</v>
       </c>
       <c r="F676" s="36" t="s">
         <v>1116</v>
       </c>
       <c r="G676" s="25"/>
       <c r="H676" s="7" t="s">
-        <v>2064</v>
+        <v>1836</v>
       </c>
       <c r="I676" s="8" t="s">
         <v>1837</v>
@@ -34427,16 +34124,16 @@
         <v>1083</v>
       </c>
       <c r="B677" s="69" t="s">
-        <v>2065</v>
+        <v>1991</v>
       </c>
       <c r="C677" s="69" t="s">
-        <v>2065</v>
+        <v>1991</v>
       </c>
       <c r="D677" s="69" t="s">
-        <v>2066</v>
+        <v>1992</v>
       </c>
       <c r="E677" s="37" t="s">
-        <v>2067</v>
+        <v>1993</v>
       </c>
       <c r="F677" s="37" t="s">
         <v>1116</v>
@@ -34445,7 +34142,7 @@
         <v>1087</v>
       </c>
       <c r="H677" s="7" t="s">
-        <v>2068</v>
+        <v>1836</v>
       </c>
       <c r="I677" s="8" t="s">
         <v>1837</v>
@@ -34468,23 +34165,23 @@
         <v>1077</v>
       </c>
       <c r="B678" s="64" t="s">
-        <v>2069</v>
+        <v>1994</v>
       </c>
       <c r="C678" s="64" t="s">
-        <v>2069</v>
+        <v>1994</v>
       </c>
       <c r="D678" s="64" t="s">
         <v>873</v>
       </c>
       <c r="E678" s="36" t="s">
-        <v>2070</v>
+        <v>1995</v>
       </c>
       <c r="F678" s="25"/>
       <c r="G678" s="36" t="s">
         <v>1455</v>
       </c>
       <c r="H678" s="7" t="s">
-        <v>2071</v>
+        <v>1836</v>
       </c>
       <c r="I678" s="8" t="s">
         <v>1837</v>
@@ -34507,16 +34204,16 @@
         <v>1107</v>
       </c>
       <c r="B679" s="69" t="s">
-        <v>2072</v>
+        <v>1996</v>
       </c>
       <c r="C679" s="69" t="s">
-        <v>2072</v>
+        <v>1996</v>
       </c>
       <c r="D679" s="69" t="s">
         <v>927</v>
       </c>
       <c r="E679" s="37" t="s">
-        <v>2073</v>
+        <v>1997</v>
       </c>
       <c r="F679" s="37" t="s">
         <v>1217</v>
@@ -34525,7 +34222,7 @@
         <v>1455</v>
       </c>
       <c r="H679" s="7" t="s">
-        <v>2074</v>
+        <v>1836</v>
       </c>
       <c r="I679" s="8" t="s">
         <v>1837</v>
@@ -34554,10 +34251,10 @@
         <v>929</v>
       </c>
       <c r="D680" s="64" t="s">
-        <v>2075</v>
+        <v>1998</v>
       </c>
       <c r="E680" s="36" t="s">
-        <v>2076</v>
+        <v>1999</v>
       </c>
       <c r="F680" s="36" t="s">
         <v>1840</v>
@@ -34566,7 +34263,7 @@
         <v>1111</v>
       </c>
       <c r="H680" s="7" t="s">
-        <v>2077</v>
+        <v>1836</v>
       </c>
       <c r="I680" s="8" t="s">
         <v>1837</v>
@@ -34589,16 +34286,16 @@
         <v>1088</v>
       </c>
       <c r="B681" s="69" t="s">
-        <v>2078</v>
+        <v>2000</v>
       </c>
       <c r="C681" s="69" t="s">
-        <v>2078</v>
+        <v>2000</v>
       </c>
       <c r="D681" s="69" t="s">
         <v>937</v>
       </c>
       <c r="E681" s="37" t="s">
-        <v>2079</v>
+        <v>2001</v>
       </c>
       <c r="F681" s="37" t="s">
         <v>1127</v>
@@ -34607,7 +34304,7 @@
         <v>1147</v>
       </c>
       <c r="H681" s="7" t="s">
-        <v>2080</v>
+        <v>1836</v>
       </c>
       <c r="I681" s="8" t="s">
         <v>1837</v>
@@ -34636,10 +34333,10 @@
         <v>936</v>
       </c>
       <c r="D682" s="64" t="s">
-        <v>2081</v>
+        <v>2002</v>
       </c>
       <c r="E682" s="36" t="s">
-        <v>2082</v>
+        <v>2003</v>
       </c>
       <c r="F682" s="36" t="s">
         <v>1441</v>
@@ -34648,7 +34345,7 @@
         <v>1111</v>
       </c>
       <c r="H682" s="7" t="s">
-        <v>2083</v>
+        <v>1836</v>
       </c>
       <c r="I682" s="8" t="s">
         <v>1837</v>
@@ -34680,7 +34377,7 @@
         <v>967</v>
       </c>
       <c r="E683" s="37" t="s">
-        <v>2084</v>
+        <v>2004</v>
       </c>
       <c r="F683" s="37" t="s">
         <v>1840</v>
@@ -34689,7 +34386,7 @@
         <v>1455</v>
       </c>
       <c r="H683" s="7" t="s">
-        <v>2085</v>
+        <v>1836</v>
       </c>
       <c r="I683" s="8" t="s">
         <v>1837</v>
@@ -34712,23 +34409,23 @@
         <v>1083</v>
       </c>
       <c r="B684" s="64" t="s">
-        <v>2086</v>
+        <v>2005</v>
       </c>
       <c r="C684" s="64" t="s">
-        <v>2086</v>
+        <v>2005</v>
       </c>
       <c r="D684" s="64" t="s">
         <v>973</v>
       </c>
       <c r="E684" s="36" t="s">
-        <v>2087</v>
+        <v>2006</v>
       </c>
       <c r="F684" s="36" t="s">
         <v>1095</v>
       </c>
       <c r="G684" s="25"/>
       <c r="H684" s="7" t="s">
-        <v>2088</v>
+        <v>1836</v>
       </c>
       <c r="I684" s="8" t="s">
         <v>1837</v>
@@ -34757,10 +34454,10 @@
         <v>984</v>
       </c>
       <c r="D685" s="69" t="s">
-        <v>2089</v>
+        <v>2007</v>
       </c>
       <c r="E685" s="37" t="s">
-        <v>2090</v>
+        <v>2008</v>
       </c>
       <c r="F685" s="37" t="s">
         <v>1441</v>
@@ -34769,7 +34466,7 @@
         <v>1087</v>
       </c>
       <c r="H685" s="7" t="s">
-        <v>2091</v>
+        <v>1836</v>
       </c>
       <c r="I685" s="8" t="s">
         <v>1837</v>
@@ -34801,14 +34498,14 @@
         <v>995</v>
       </c>
       <c r="E686" s="36" t="s">
-        <v>2092</v>
+        <v>2009</v>
       </c>
       <c r="F686" s="25"/>
       <c r="G686" s="36" t="s">
         <v>1455</v>
       </c>
       <c r="H686" s="7" t="s">
-        <v>2093</v>
+        <v>1836</v>
       </c>
       <c r="I686" s="8" t="s">
         <v>1837</v>
@@ -34831,16 +34528,16 @@
         <v>1107</v>
       </c>
       <c r="B687" s="69" t="s">
-        <v>2094</v>
+        <v>2010</v>
       </c>
       <c r="C687" s="69" t="s">
-        <v>2094</v>
+        <v>2010</v>
       </c>
       <c r="D687" s="69" t="s">
-        <v>2095</v>
+        <v>2011</v>
       </c>
       <c r="E687" s="37" t="s">
-        <v>2096</v>
+        <v>2012</v>
       </c>
       <c r="F687" s="37" t="s">
         <v>1840</v>
@@ -34849,7 +34546,7 @@
         <v>1123</v>
       </c>
       <c r="H687" s="7" t="s">
-        <v>2097</v>
+        <v>1836</v>
       </c>
       <c r="I687" s="8" t="s">
         <v>1837</v>
@@ -34878,10 +34575,10 @@
         <v>1016</v>
       </c>
       <c r="D688" s="64" t="s">
-        <v>2098</v>
+        <v>2013</v>
       </c>
       <c r="E688" s="36" t="s">
-        <v>2099</v>
+        <v>2014</v>
       </c>
       <c r="F688" s="36" t="s">
         <v>1086</v>
@@ -34890,7 +34587,7 @@
         <v>1087</v>
       </c>
       <c r="H688" s="7" t="s">
-        <v>2100</v>
+        <v>1836</v>
       </c>
       <c r="I688" s="8" t="s">
         <v>1837</v>
@@ -34910,22 +34607,22 @@
     </row>
     <row r="689" ht="12.75" customHeight="1">
       <c r="A689" s="68" t="s">
-        <v>2101</v>
+        <v>2015</v>
       </c>
       <c r="B689" s="69" t="s">
         <v>1040</v>
       </c>
       <c r="C689" s="69" t="s">
-        <v>2102</v>
+        <v>2016</v>
       </c>
       <c r="D689" s="69" t="s">
-        <v>2103</v>
+        <v>2017</v>
       </c>
       <c r="E689" s="30"/>
       <c r="F689" s="30"/>
       <c r="G689" s="30"/>
       <c r="H689" s="7" t="s">
-        <v>2104</v>
+        <v>1836</v>
       </c>
       <c r="I689" s="8" t="s">
         <v>1837</v>
@@ -34948,23 +34645,23 @@
         <v>1077</v>
       </c>
       <c r="B690" s="64" t="s">
-        <v>2105</v>
+        <v>2018</v>
       </c>
       <c r="C690" s="64" t="s">
-        <v>2105</v>
+        <v>2018</v>
       </c>
       <c r="D690" s="64" t="s">
         <v>1667</v>
       </c>
       <c r="E690" s="36" t="s">
-        <v>2106</v>
+        <v>2019</v>
       </c>
       <c r="F690" s="25"/>
       <c r="G690" s="36" t="s">
         <v>1455</v>
       </c>
       <c r="H690" s="7" t="s">
-        <v>2107</v>
+        <v>1836</v>
       </c>
       <c r="I690" s="8" t="s">
         <v>1837</v>
@@ -34987,23 +34684,23 @@
         <v>1112</v>
       </c>
       <c r="B691" s="69" t="s">
-        <v>2108</v>
+        <v>2020</v>
       </c>
       <c r="C691" s="69" t="s">
-        <v>2109</v>
+        <v>2021</v>
       </c>
       <c r="D691" s="69" t="s">
-        <v>2110</v>
+        <v>2022</v>
       </c>
       <c r="E691" s="37" t="s">
-        <v>2111</v>
+        <v>2023</v>
       </c>
       <c r="F691" s="37" t="s">
         <v>1095</v>
       </c>
       <c r="G691" s="30"/>
       <c r="H691" s="7" t="s">
-        <v>2112</v>
+        <v>1836</v>
       </c>
       <c r="I691" s="8" t="s">
         <v>1837</v>
@@ -35026,25 +34723,25 @@
         <v>1107</v>
       </c>
       <c r="B692" s="64" t="s">
-        <v>2113</v>
+        <v>2024</v>
       </c>
       <c r="C692" s="64" t="s">
-        <v>2113</v>
+        <v>2024</v>
       </c>
       <c r="D692" s="83" t="s">
-        <v>2114</v>
+        <v>2025</v>
       </c>
       <c r="E692" s="36" t="s">
-        <v>2115</v>
+        <v>2026</v>
       </c>
       <c r="F692" s="36" t="s">
-        <v>1881</v>
+        <v>1867</v>
       </c>
       <c r="G692" s="36" t="s">
         <v>1111</v>
       </c>
       <c r="H692" s="7" t="s">
-        <v>2116</v>
+        <v>1836</v>
       </c>
       <c r="I692" s="8" t="s">
         <v>1837</v>
@@ -35067,16 +34764,16 @@
         <v>1107</v>
       </c>
       <c r="B693" s="69" t="s">
-        <v>2117</v>
+        <v>2027</v>
       </c>
       <c r="C693" s="69" t="s">
-        <v>2117</v>
+        <v>2027</v>
       </c>
       <c r="D693" s="69" t="s">
-        <v>2118</v>
+        <v>2028</v>
       </c>
       <c r="E693" s="37" t="s">
-        <v>2119</v>
+        <v>2029</v>
       </c>
       <c r="F693" s="37" t="s">
         <v>1840</v>
@@ -35085,7 +34782,7 @@
         <v>1111</v>
       </c>
       <c r="H693" s="7" t="s">
-        <v>2120</v>
+        <v>1836</v>
       </c>
       <c r="I693" s="8" t="s">
         <v>1837</v>
@@ -35108,23 +34805,23 @@
         <v>1083</v>
       </c>
       <c r="B694" s="64" t="s">
-        <v>2121</v>
+        <v>2030</v>
       </c>
       <c r="C694" s="64" t="s">
-        <v>2121</v>
+        <v>2030</v>
       </c>
       <c r="D694" s="64" t="s">
-        <v>2122</v>
+        <v>2031</v>
       </c>
       <c r="E694" s="36" t="s">
-        <v>2123</v>
+        <v>2032</v>
       </c>
       <c r="F694" s="36" t="s">
         <v>1095</v>
       </c>
       <c r="G694" s="25"/>
       <c r="H694" s="7" t="s">
-        <v>2124</v>
+        <v>1836</v>
       </c>
       <c r="I694" s="8" t="s">
         <v>1837</v>
@@ -35147,23 +34844,23 @@
         <v>1077</v>
       </c>
       <c r="B695" s="69" t="s">
-        <v>2125</v>
+        <v>2033</v>
       </c>
       <c r="C695" s="69" t="s">
-        <v>2125</v>
+        <v>2033</v>
       </c>
       <c r="D695" s="69" t="s">
-        <v>2126</v>
+        <v>2034</v>
       </c>
       <c r="E695" s="37" t="s">
-        <v>2127</v>
+        <v>2035</v>
       </c>
       <c r="F695" s="30"/>
       <c r="G695" s="37" t="s">
         <v>1147</v>
       </c>
       <c r="H695" s="7" t="s">
-        <v>2128</v>
+        <v>1836</v>
       </c>
       <c r="I695" s="8" t="s">
         <v>1837</v>
@@ -35186,25 +34883,25 @@
         <v>1107</v>
       </c>
       <c r="B696" s="64" t="s">
-        <v>2129</v>
+        <v>2036</v>
       </c>
       <c r="C696" s="64" t="s">
-        <v>2129</v>
+        <v>2036</v>
       </c>
       <c r="D696" s="64" t="s">
-        <v>2130</v>
+        <v>2037</v>
       </c>
       <c r="E696" s="36" t="s">
-        <v>2131</v>
+        <v>2038</v>
       </c>
       <c r="F696" s="36" t="s">
         <v>1217</v>
       </c>
       <c r="G696" s="36" t="s">
-        <v>2132</v>
+        <v>2039</v>
       </c>
       <c r="H696" s="7" t="s">
-        <v>2133</v>
+        <v>1836</v>
       </c>
       <c r="I696" s="8" t="s">
         <v>1837</v>
@@ -35227,16 +34924,16 @@
         <v>1148</v>
       </c>
       <c r="B697" s="69" t="s">
-        <v>2134</v>
+        <v>2040</v>
       </c>
       <c r="C697" s="69" t="s">
-        <v>2134</v>
+        <v>2040</v>
       </c>
       <c r="D697" s="69" t="s">
-        <v>2135</v>
+        <v>2041</v>
       </c>
       <c r="E697" s="37" t="s">
-        <v>2136</v>
+        <v>2042</v>
       </c>
       <c r="F697" s="37" t="s">
         <v>1441</v>
@@ -35245,7 +34942,7 @@
         <v>1123</v>
       </c>
       <c r="H697" s="7" t="s">
-        <v>2137</v>
+        <v>1836</v>
       </c>
       <c r="I697" s="8" t="s">
         <v>1837</v>
@@ -35268,16 +34965,16 @@
         <v>1083</v>
       </c>
       <c r="B698" s="64" t="s">
-        <v>2138</v>
+        <v>2043</v>
       </c>
       <c r="C698" s="64" t="s">
-        <v>2138</v>
+        <v>2043</v>
       </c>
       <c r="D698" s="64" t="s">
         <v>1825</v>
       </c>
       <c r="E698" s="36" t="s">
-        <v>2139</v>
+        <v>2044</v>
       </c>
       <c r="F698" s="36" t="s">
         <v>1095</v>
@@ -35286,7 +34983,7 @@
         <v>1087</v>
       </c>
       <c r="H698" s="7" t="s">
-        <v>2140</v>
+        <v>1836</v>
       </c>
       <c r="I698" s="8" t="s">
         <v>1837</v>
@@ -35309,23 +35006,23 @@
         <v>1077</v>
       </c>
       <c r="B699" s="69" t="s">
-        <v>2141</v>
+        <v>2045</v>
       </c>
       <c r="C699" s="69" t="s">
-        <v>2141</v>
+        <v>2045</v>
       </c>
       <c r="D699" s="69" t="s">
-        <v>2142</v>
+        <v>2046</v>
       </c>
       <c r="E699" s="37" t="s">
-        <v>2143</v>
+        <v>2047</v>
       </c>
       <c r="F699" s="30"/>
       <c r="G699" s="37" t="s">
         <v>1133</v>
       </c>
       <c r="H699" s="7" t="s">
-        <v>2144</v>
+        <v>1836</v>
       </c>
       <c r="I699" s="8" t="s">
         <v>1837</v>
@@ -35348,16 +35045,16 @@
         <v>1148</v>
       </c>
       <c r="B700" s="64" t="s">
-        <v>2145</v>
+        <v>2048</v>
       </c>
       <c r="C700" s="64" t="s">
-        <v>2145</v>
+        <v>2048</v>
       </c>
       <c r="D700" s="64" t="s">
-        <v>2146</v>
+        <v>2049</v>
       </c>
       <c r="E700" s="36" t="s">
-        <v>2147</v>
+        <v>2050</v>
       </c>
       <c r="F700" s="36" t="s">
         <v>1441</v>
@@ -35366,7 +35063,7 @@
         <v>1087</v>
       </c>
       <c r="H700" s="7" t="s">
-        <v>2148</v>
+        <v>1836</v>
       </c>
       <c r="I700" s="8" t="s">
         <v>1837</v>
@@ -35389,21 +35086,21 @@
         <v>1077</v>
       </c>
       <c r="B701" s="69" t="s">
-        <v>2149</v>
+        <v>2051</v>
       </c>
       <c r="C701" s="69" t="s">
-        <v>2149</v>
+        <v>2051</v>
       </c>
       <c r="D701" s="69" t="s">
-        <v>2150</v>
+        <v>2052</v>
       </c>
       <c r="E701" s="37" t="s">
-        <v>2151</v>
+        <v>2053</v>
       </c>
       <c r="F701" s="30"/>
       <c r="G701" s="30"/>
       <c r="H701" s="7" t="s">
-        <v>2152</v>
+        <v>1836</v>
       </c>
       <c r="I701" s="8" t="s">
         <v>1837</v>
@@ -35426,16 +35123,16 @@
         <v>1148</v>
       </c>
       <c r="B702" s="64" t="s">
-        <v>2153</v>
+        <v>2054</v>
       </c>
       <c r="C702" s="64" t="s">
-        <v>2153</v>
+        <v>2054</v>
       </c>
       <c r="D702" s="64" t="s">
-        <v>2154</v>
+        <v>2055</v>
       </c>
       <c r="E702" s="36" t="s">
-        <v>2155</v>
+        <v>2056</v>
       </c>
       <c r="F702" s="36" t="s">
         <v>1441</v>
@@ -35444,7 +35141,7 @@
         <v>1087</v>
       </c>
       <c r="H702" s="7" t="s">
-        <v>2156</v>
+        <v>1836</v>
       </c>
       <c r="I702" s="8" t="s">
         <v>1837</v>
@@ -35464,13 +35161,13 @@
     </row>
     <row r="703" ht="12.75" customHeight="1">
       <c r="A703" s="68" t="s">
-        <v>2157</v>
+        <v>2057</v>
       </c>
       <c r="B703" s="69" t="s">
-        <v>2158</v>
+        <v>2058</v>
       </c>
       <c r="C703" s="69" t="s">
-        <v>2159</v>
+        <v>2059</v>
       </c>
       <c r="D703" s="69" t="s">
         <v>1101</v>
@@ -35479,7 +35176,7 @@
       <c r="F703" s="30"/>
       <c r="G703" s="30"/>
       <c r="H703" s="7" t="s">
-        <v>2160</v>
+        <v>1836</v>
       </c>
       <c r="I703" s="8" t="s">
         <v>1837</v>

</xml_diff>